<commit_message>
Agregar hojas Gastos Inicio y Gastos Mensuales con prioridades
Gastos Inicio alimenta la inversion inicial y calcula la caja recomendada
para partir; Gastos Mensuales alimenta plataforma, marketing y otros en Supuestos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FyrtynBGssxjxAFxFhXjrS
</commit_message>
<xml_diff>
--- a/Viabilidad_Academia_LoL.xlsx
+++ b/Viabilidad_Academia_LoL.xlsx
@@ -10,9 +10,11 @@
   <sheets>
     <sheet name="Supuestos" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Inversion" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Flujo de Caja" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Indicadores" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Valor Ganado" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Gastos Inicio" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Gastos Mensuales" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Flujo de Caja" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Indicadores" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Valor Ganado" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="239">
   <si>
     <t xml:space="preserve">Academia de League of Legends - Supuestos del modelo</t>
   </si>
@@ -95,19 +97,19 @@
     <t xml:space="preserve">Plataforma y software mensual (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Supuesto: Discord Nitro, hosting web, herramientas VOD</t>
+    <t xml:space="preserve">Viene de la hoja Gastos Mensuales (categoria Plataforma, solo lo incluido)</t>
   </si>
   <si>
     <t xml:space="preserve">Marketing mensual (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Supuesto: anuncios en redes / creadores</t>
+    <t xml:space="preserve">Viene de la hoja Gastos Mensuales (categoria Marketing, solo lo incluido)</t>
   </si>
   <si>
     <t xml:space="preserve">Otros gastos mensuales (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Supuesto: administracion, varios</t>
+    <t xml:space="preserve">Viene de la hoja Gastos Mensuales (categoria Otros, solo lo incluido)</t>
   </si>
   <si>
     <t xml:space="preserve">Tasa de impuesto sobre utilidad</t>
@@ -158,7 +160,7 @@
     <t xml:space="preserve">Inversion inicial (mes 0)</t>
   </si>
   <si>
-    <t xml:space="preserve">Edita los montos en azul. Los imprevistos se calculan como % del subtotal.</t>
+    <t xml:space="preserve">Los montos vienen de la hoja Gastos Inicio (solo lo marcado 'Si'). Edita alli.</t>
   </si>
   <si>
     <t xml:space="preserve">Concepto</t>
@@ -170,37 +172,259 @@
     <t xml:space="preserve">Comentario</t>
   </si>
   <si>
+    <t xml:space="preserve">Gastos vitales incluidos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viene de la hoja Gastos Inicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gastos importantes incluidos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gastos opcionales incluidos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% imprevistos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: colchon para gastos no previstos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imprevistos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INVERSION INICIAL TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gastos de inicio - que es vital para partir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clasifica cada gasto (Vital / Importante / Opcional) y marca Si/No en 'Incluir'. Solo lo marcado 'Si' suma a la inversion inicial. Edita las celdas amarillas; agrega gastos en las filas vacias.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gasto de inicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prioridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo estimado (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incluir (Si/No)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monto incluido (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branding (logo, overlays, redes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dato del usuario (antes en hoja Inversion)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campana de marketing de lanzamiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servidor de Discord (canales, roles, bots gratuitos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: se puede armar sin costo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuenta bancaria para recibir transferencias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: cuenta vista / digital sin costo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Material de clases (guias, plantillas de VOD review)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Importante</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: lo crean los coaches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pagina web / landing de inscripcion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: dominio + landing simple. Alternativa gratis: Linktree / formulario</t>
+  </si>
+  <si>
     <t xml:space="preserve">Constitucion legal y tramites</t>
   </si>
   <si>
-    <t xml:space="preserve">Pagina web / landing de inscripcion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Branding (logo, overlays, redes)</t>
+    <t xml:space="preserve">Supuesto: formalizar cuando haya ingresos estables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Licencias y herramientas iniciales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opcional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: herramientas de analisis / edicion</t>
   </si>
   <si>
     <t xml:space="preserve">Equipo de streaming (microfono, camara)</t>
   </si>
   <si>
-    <t xml:space="preserve">Licencias y herramientas iniciales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campana de marketing de lanzamiento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subtotal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% imprevistos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supuesto: colchon para gastos no previstos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Imprevistos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INVERSION INICIAL TOTAL</t>
+    <t xml:space="preserve">Supuesto: coaches usan su propio equipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sorteo de lanzamiento (RP / skins)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: gancho para primeros alumnos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resumen por prioridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incluido (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuanto dinero tener para partir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inversion inicial total (incluido + imprevistos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viene de la hoja Inversion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gasto mensual total (coaches + gastos incluidos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viene de la hoja Gastos Mensuales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meses de gastos como reserva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: colchon por si entran menos alumnos o pagan tarde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fondo de reserva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gasto mensual x meses de reserva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAJA RECOMENDADA PARA PARTIR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inversion inicial + fondo de reserva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gastos mensuales - en que invertir cada mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cada gasto tiene categoria (alimenta la hoja Supuestos) y prioridad. Solo lo marcado 'Si' entra al flujo de caja. Los sueldos de coaches se calculan en Supuestos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gasto mensual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo mensual (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discord Nitro / boost del servidor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plataforma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dato del usuario: plataforma = 10 USD/mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Herramienta de analisis de partidas / VOD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dominio y hosting web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: solo si hay pagina web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anuncios en redes (TikTok / Instagram)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dato del usuario: marketing = 80 USD/mes (repartido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colaboraciones con streamers / creadores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Premios torneos internos (RP / skins)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: retencion de alumnos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internet y servicios (proporcion)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Otros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dato del usuario: otros = 30 USD/mes (repartido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Administracion y contabilidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL GASTOS (sin sueldos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resumen mensual (incluido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USD / mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sueldos de coaches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viene de Supuestos (coaches que cobran x sueldo x horas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GASTO MENSUAL TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por prioridad (incluido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingreso mensual esperado (mes 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingreso - gasto mensual total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si es negativo, recorta primero lo Opcional y luego lo Importante</t>
   </si>
   <si>
     <t xml:space="preserve">Flujo de caja proyectado - 6 meses (USD)</t>
@@ -525,15 +749,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="166" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="167" formatCode="0.0%;\(0.0%\);\-"/>
     <numFmt numFmtId="168" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="169" formatCode="0.000%"/>
-    <numFmt numFmtId="170" formatCode="0"/>
-    <numFmt numFmtId="171" formatCode="0.00"/>
+    <numFmt numFmtId="170" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
+    <numFmt numFmtId="171" formatCode="0"/>
+    <numFmt numFmtId="172" formatCode="0.00"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -596,15 +821,15 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="11"/>
+      <color rgb="FF008000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF008000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -711,92 +936,140 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="50">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -804,11 +1077,43 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -816,19 +1121,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -841,6 +1146,29 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFE699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -877,12 +1205,12 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFE2EFDA"/>
+      <rgbColor rgb="FFFFE699"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFF8CBAD"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -939,8 +1267,8 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.22158987929097"/>
-          <c:y val="0.0310077519379845"/>
+          <c:x val="0.221634162256217"/>
+          <c:y val="0.0311366762535951"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -1071,11 +1399,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="65207347"/>
-        <c:axId val="55858119"/>
+        <c:axId val="14966397"/>
+        <c:axId val="97645602"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="65207347"/>
+        <c:axId val="14966397"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1141,7 +1469,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55858119"/>
+        <c:crossAx val="97645602"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1149,7 +1477,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="55858119"/>
+        <c:axId val="97645602"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1225,7 +1553,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65207347"/>
+        <c:crossAx val="14966397"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1264,9 +1592,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>136080</xdr:colOff>
+      <xdr:colOff>135720</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>145440</xdr:rowOff>
+      <xdr:rowOff>145080</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1275,7 +1603,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="1380960" y="3667320"/>
-        <a:ext cx="9930960" cy="2878920"/>
+        <a:ext cx="9930600" cy="2878560"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1471,250 +1799,253 @@
   <dimension ref="A1:C24"/>
   <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="8" t="n">
         <v>0.15</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="B12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="9" t="n">
+        <f aca="false">'Gastos Mensuales'!$F$21</f>
         <v>10</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="9" t="n">
+        <f aca="false">'Gastos Mensuales'!$F$22</f>
         <v>80</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="9" t="n">
+        <f aca="false">'Gastos Mensuales'!$F$23</f>
         <v>30</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="7" t="n">
+      <c r="B16" s="8" t="n">
         <v>0.27</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="7" t="n">
+      <c r="B17" s="8" t="n">
         <v>0.12</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="11" t="n">
         <f aca="false">(1+B17)^(1/12)-1</f>
         <v>0.00948879293458305</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B21" s="12" t="n">
         <f aca="false">B7*B8</f>
         <v>15</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B22" s="12" t="n">
+      <c r="B22" s="13" t="n">
         <f aca="false">(B8-B9)*B10*B11</f>
         <v>40</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B23" s="12" t="n">
+      <c r="B23" s="13" t="n">
         <f aca="false">B22+B13+B14+B15</f>
         <v>160</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B24" s="13" t="n">
+      <c r="B24" s="14" t="n">
         <f aca="false">B4*(1-B12)</f>
         <v>15</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="3" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1740,132 +2071,119 @@
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="B4" s="15" t="n">
+        <f aca="false">'Gastos Inicio'!$E$23</f>
+        <v>80</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B6" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="B5" s="15" t="n">
+        <f aca="false">'Gastos Inicio'!$E$24</f>
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="B6" s="15" t="n">
+        <f aca="false">'Gastos Inicio'!$E$25</f>
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="18"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="18"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="18"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="B8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B9" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="20" t="n">
         <f aca="false">SUM(B4:B9)</f>
         <v>80</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="7" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="13" t="n">
         <f aca="false">B10*B11</f>
         <v>8</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13" s="17" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="22" t="n">
         <f aca="false">B10+B12</f>
         <v>88</v>
       </c>
@@ -1889,531 +2207,1577 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="62"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="26" t="n">
+        <v>50</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="E5" s="27" t="n">
+        <f aca="false">IF(D5="Si",N(C5),0)</f>
+        <v>50</v>
+      </c>
+      <c r="F5" s="28" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="26" t="n">
+        <v>30</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="E6" s="27" t="n">
+        <f aca="false">IF(D6="Si",N(C6),0)</f>
+        <v>30</v>
+      </c>
+      <c r="F6" s="28" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="E7" s="27" t="n">
+        <f aca="false">IF(D7="Si",N(C7),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="28" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" s="27" t="n">
+        <f aca="false">IF(D8="Si",N(C8),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="28" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="24" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="E9" s="27" t="n">
+        <f aca="false">IF(D9="Si",N(C9),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="28" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="E10" s="27" t="n">
+        <f aca="false">IF(D10="Si",N(C10),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="28" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="C11" s="26" t="n">
+        <v>300</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11" s="27" t="n">
+        <f aca="false">IF(D11="Si",N(C11),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="28" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="C12" s="26" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="E12" s="27" t="n">
+        <f aca="false">IF(D12="Si",N(C12),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="28" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" s="26" t="n">
+        <v>150</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="E13" s="27" t="n">
+        <f aca="false">IF(D13="Si",N(C13),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="B14" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" s="26" t="n">
+        <v>20</v>
+      </c>
+      <c r="D14" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" s="27" t="n">
+        <f aca="false">IF(D14="Si",N(C14),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="24"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="27" t="n">
+        <f aca="false">IF(D15="Si",N(C15),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="28"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="24"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="27" t="n">
+        <f aca="false">IF(D16="Si",N(C16),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F16" s="28"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="24"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="27" t="n">
+        <f aca="false">IF(D17="Si",N(C17),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="28"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="24"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="27" t="n">
+        <f aca="false">IF(D18="Si",N(C18),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F18" s="28"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="24"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="27" t="n">
+        <f aca="false">IF(D19="Si",N(C19),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="28"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="C20" s="30" t="n">
+        <f aca="false">SUM(C5:C19)</f>
+        <v>700</v>
+      </c>
+      <c r="E20" s="30" t="n">
+        <f aca="false">SUM(E5:E19)</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="31" t="s">
+        <v>89</v>
+      </c>
+      <c r="B22" s="31"/>
+      <c r="C22" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="F22" s="31"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="32" t="s">
+        <v>65</v>
+      </c>
+      <c r="C23" s="27" t="n">
+        <f aca="false">SUMIFS($C$5:$C$19,$B$5:$B$19,"Vital")</f>
+        <v>80</v>
+      </c>
+      <c r="E23" s="27" t="n">
+        <f aca="false">SUMIFS($E$5:$E$19,$B$5:$B$19,"Vital")</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="C24" s="27" t="n">
+        <f aca="false">SUMIFS($C$5:$C$19,$B$5:$B$19,"Importante")</f>
+        <v>400</v>
+      </c>
+      <c r="E24" s="27" t="n">
+        <f aca="false">SUMIFS($E$5:$E$19,$B$5:$B$19,"Importante")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="C25" s="27" t="n">
+        <f aca="false">SUMIFS($C$5:$C$19,$B$5:$B$19,"Opcional")</f>
+        <v>220</v>
+      </c>
+      <c r="E25" s="27" t="n">
+        <f aca="false">SUMIFS($E$5:$E$19,$B$5:$B$19,"Opcional")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="33" t="s">
+        <v>91</v>
+      </c>
+      <c r="B27" s="34"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="34"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="32" t="s">
+        <v>92</v>
+      </c>
+      <c r="C28" s="35" t="n">
+        <f aca="false">Inversion!$B$13</f>
+        <v>88</v>
+      </c>
+      <c r="D28" s="28" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="32" t="s">
+        <v>94</v>
+      </c>
+      <c r="C29" s="35" t="n">
+        <f aca="false">'Gastos Mensuales'!$F$25</f>
+        <v>160</v>
+      </c>
+      <c r="D29" s="28" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="C30" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="28" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="C31" s="27" t="n">
+        <f aca="false">C29*C30</f>
+        <v>160</v>
+      </c>
+      <c r="D31" s="28" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="37" t="s">
+        <v>100</v>
+      </c>
+      <c r="C32" s="30" t="n">
+        <f aca="false">C28+C31</f>
+        <v>248</v>
+      </c>
+      <c r="D32" s="28" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B5:B19">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"Vital"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Importante"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>"Opcional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A23">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"Vital"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Importante"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>"Opcional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A24">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"Vital"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Importante"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>"Opcional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A25">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"Vital"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Importante"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="13" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>"Opcional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B19" type="list">
+      <formula1>"Vital,Importante,Opcional"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D19" type="list">
+      <formula1>"Si,No"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G32"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="55"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="F5" s="27" t="n">
+        <f aca="false">IF(E5="Si",N(D5),0)</f>
+        <v>10</v>
+      </c>
+      <c r="G5" s="28" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="F6" s="27" t="n">
+        <f aca="false">IF(E6="Si",N(D6),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="28" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="F7" s="27" t="n">
+        <f aca="false">IF(E7="Si",N(D7),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="28" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>50</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" s="27" t="n">
+        <f aca="false">IF(E8="Si",N(D8),0)</f>
+        <v>50</v>
+      </c>
+      <c r="G8" s="28" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>30</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="F9" s="27" t="n">
+        <f aca="false">IF(E9="Si",N(D9),0)</f>
+        <v>30</v>
+      </c>
+      <c r="G9" s="28" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="24" t="s">
+        <v>117</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="D10" s="26" t="n">
+        <v>20</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="F10" s="27" t="n">
+        <f aca="false">IF(E10="Si",N(D10),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="28" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="26" t="n">
+        <v>20</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="F11" s="27" t="n">
+        <f aca="false">IF(E11="Si",N(D11),0)</f>
+        <v>20</v>
+      </c>
+      <c r="G11" s="28" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="B12" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="E12" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="F12" s="27" t="n">
+        <f aca="false">IF(E12="Si",N(D12),0)</f>
+        <v>10</v>
+      </c>
+      <c r="G12" s="28" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="24"/>
+      <c r="B13" s="25"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="27" t="n">
+        <f aca="false">IF(E13="Si",N(D13),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="28"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="24"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="27" t="n">
+        <f aca="false">IF(E14="Si",N(D14),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="28"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="24"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="27" t="n">
+        <f aca="false">IF(E15="Si",N(D15),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="28"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="24"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="27" t="n">
+        <f aca="false">IF(E16="Si",N(D16),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="28"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="24"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="27" t="n">
+        <f aca="false">IF(E17="Si",N(D17),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="28"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="D18" s="30" t="n">
+        <f aca="false">SUM(D5:D17)</f>
+        <v>160</v>
+      </c>
+      <c r="F18" s="30" t="n">
+        <f aca="false">SUM(F5:F17)</f>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="31" t="s">
+        <v>124</v>
+      </c>
+      <c r="B20" s="31"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="G20" s="31"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="F21" s="27" t="n">
+        <f aca="false">SUMIFS($F$5:$F$17,$B$5:$B$17,"Plataforma")</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="32" t="s">
+        <v>114</v>
+      </c>
+      <c r="F22" s="27" t="n">
+        <f aca="false">SUMIFS($F$5:$F$17,$B$5:$B$17,"Marketing")</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="F23" s="27" t="n">
+        <f aca="false">SUMIFS($F$5:$F$17,$B$5:$B$17,"Otros")</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="32" t="s">
+        <v>126</v>
+      </c>
+      <c r="F24" s="35" t="n">
+        <f aca="false">Supuestos!$B$22</f>
+        <v>40</v>
+      </c>
+      <c r="G24" s="28" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="F25" s="30" t="n">
+        <f aca="false">SUM(F21:F24)</f>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="B27" s="31"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="G27" s="31"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="32" t="s">
+        <v>65</v>
+      </c>
+      <c r="F28" s="27" t="n">
+        <f aca="false">SUMIFS($F$5:$F$17,$C$5:$C$17,"Vital")</f>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="F29" s="27" t="n">
+        <f aca="false">SUMIFS($F$5:$F$17,$C$5:$C$17,"Importante")</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="F30" s="27" t="n">
+        <f aca="false">SUMIFS($F$5:$F$17,$C$5:$C$17,"Opcional")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="F31" s="35" t="n">
+        <f aca="false">'Flujo de Caja'!$C$5</f>
+        <v>225</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="29" t="s">
+        <v>131</v>
+      </c>
+      <c r="F32" s="30" t="n">
+        <f aca="false">F31-F25</f>
+        <v>65</v>
+      </c>
+      <c r="G32" s="28" t="s">
+        <v>132</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C5:C17">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"Vital"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Importante"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>"Opcional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A28">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"Vital"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Importante"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>"Opcional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A29">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"Vital"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Importante"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>"Opcional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A30">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"Vital"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Importante"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="13" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>"Opcional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B17" type="list">
+      <formula1>"Plataforma,Marketing,Otros"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C17" type="list">
+      <formula1>"Vital,Importante,Opcional"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E17" type="list">
+      <formula1>"Si,No"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:H20"/>
   <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="1" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A1" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" s="18" t="n">
+      <c r="B3" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="B4" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="39" t="n">
         <f aca="false">MIN(Supuestos!$B$21,Supuestos!$B$5)</f>
         <v>15</v>
       </c>
-      <c r="D4" s="18" t="n">
+      <c r="D4" s="39" t="n">
         <f aca="false">MIN(Supuestos!$B$21,ROUND(C4*(1+Supuestos!$B$6),0))</f>
         <v>15</v>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="39" t="n">
         <f aca="false">MIN(Supuestos!$B$21,ROUND(D4*(1+Supuestos!$B$6),0))</f>
         <v>15</v>
       </c>
-      <c r="F4" s="18" t="n">
+      <c r="F4" s="39" t="n">
         <f aca="false">MIN(Supuestos!$B$21,ROUND(E4*(1+Supuestos!$B$6),0))</f>
         <v>15</v>
       </c>
-      <c r="G4" s="18" t="n">
+      <c r="G4" s="39" t="n">
         <f aca="false">MIN(Supuestos!$B$21,ROUND(F4*(1+Supuestos!$B$6),0))</f>
         <v>15</v>
       </c>
-      <c r="H4" s="18" t="n">
+      <c r="H4" s="39" t="n">
         <f aca="false">MIN(Supuestos!$B$21,ROUND(G4*(1+Supuestos!$B$6),0))</f>
         <v>15</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="19" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="9" t="n">
         <f aca="false">C4*Supuestos!$B$4</f>
         <v>225</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="9" t="n">
         <f aca="false">D4*Supuestos!$B$4</f>
         <v>225</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="9" t="n">
         <f aca="false">E4*Supuestos!$B$4</f>
         <v>225</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="9" t="n">
         <f aca="false">F4*Supuestos!$B$4</f>
         <v>225</v>
       </c>
-      <c r="G5" s="19" t="n">
+      <c r="G5" s="9" t="n">
         <f aca="false">G4*Supuestos!$B$4</f>
         <v>225</v>
       </c>
-      <c r="H5" s="19" t="n">
+      <c r="H5" s="9" t="n">
         <f aca="false">H4*Supuestos!$B$4</f>
         <v>225</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="19" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="B6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="9" t="n">
         <f aca="false">-C5*Supuestos!$B$12</f>
         <v>-0</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="9" t="n">
         <f aca="false">-D5*Supuestos!$B$12</f>
         <v>-0</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="9" t="n">
         <f aca="false">-E5*Supuestos!$B$12</f>
         <v>-0</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="9" t="n">
         <f aca="false">-F5*Supuestos!$B$12</f>
         <v>-0</v>
       </c>
-      <c r="G6" s="19" t="n">
+      <c r="G6" s="9" t="n">
         <f aca="false">-G5*Supuestos!$B$12</f>
         <v>-0</v>
       </c>
-      <c r="H6" s="19" t="n">
+      <c r="H6" s="9" t="n">
         <f aca="false">-H5*Supuestos!$B$12</f>
         <v>-0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="B7" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="12" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="40" t="s">
+        <v>144</v>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="13" t="n">
         <f aca="false">C5+C6</f>
         <v>225</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="13" t="n">
         <f aca="false">D5+D6</f>
         <v>225</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="13" t="n">
         <f aca="false">E5+E6</f>
         <v>225</v>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F7" s="13" t="n">
         <f aca="false">F5+F6</f>
         <v>225</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="13" t="n">
         <f aca="false">G5+G6</f>
         <v>225</v>
       </c>
-      <c r="H7" s="12" t="n">
+      <c r="H7" s="13" t="n">
         <f aca="false">H5+H6</f>
         <v>225</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="19" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="B8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="9" t="n">
         <f aca="false">-Supuestos!$B$22</f>
         <v>-40</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="9" t="n">
         <f aca="false">-Supuestos!$B$22</f>
         <v>-40</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="9" t="n">
         <f aca="false">-Supuestos!$B$22</f>
         <v>-40</v>
       </c>
-      <c r="F8" s="19" t="n">
+      <c r="F8" s="9" t="n">
         <f aca="false">-Supuestos!$B$22</f>
         <v>-40</v>
       </c>
-      <c r="G8" s="19" t="n">
+      <c r="G8" s="9" t="n">
         <f aca="false">-Supuestos!$B$22</f>
         <v>-40</v>
       </c>
-      <c r="H8" s="19" t="n">
+      <c r="H8" s="9" t="n">
         <f aca="false">-Supuestos!$B$22</f>
         <v>-40</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B9" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="19" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="9" t="n">
         <f aca="false">-Supuestos!$B$13</f>
         <v>-10</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="9" t="n">
         <f aca="false">-Supuestos!$B$13</f>
         <v>-10</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="9" t="n">
         <f aca="false">-Supuestos!$B$13</f>
         <v>-10</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="9" t="n">
         <f aca="false">-Supuestos!$B$13</f>
         <v>-10</v>
       </c>
-      <c r="G9" s="19" t="n">
+      <c r="G9" s="9" t="n">
         <f aca="false">-Supuestos!$B$13</f>
         <v>-10</v>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="H9" s="9" t="n">
         <f aca="false">-Supuestos!$B$13</f>
         <v>-10</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="19" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="B10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="9" t="n">
         <f aca="false">-Supuestos!$B$14</f>
         <v>-80</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="9" t="n">
         <f aca="false">-Supuestos!$B$14</f>
         <v>-80</v>
       </c>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="9" t="n">
         <f aca="false">-Supuestos!$B$14</f>
         <v>-80</v>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="9" t="n">
         <f aca="false">-Supuestos!$B$14</f>
         <v>-80</v>
       </c>
-      <c r="G10" s="19" t="n">
+      <c r="G10" s="9" t="n">
         <f aca="false">-Supuestos!$B$14</f>
         <v>-80</v>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="H10" s="9" t="n">
         <f aca="false">-Supuestos!$B$14</f>
         <v>-80</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B11" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="19" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="B11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="9" t="n">
         <f aca="false">-Supuestos!$B$15</f>
         <v>-30</v>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="9" t="n">
         <f aca="false">-Supuestos!$B$15</f>
         <v>-30</v>
       </c>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="9" t="n">
         <f aca="false">-Supuestos!$B$15</f>
         <v>-30</v>
       </c>
-      <c r="F11" s="19" t="n">
+      <c r="F11" s="9" t="n">
         <f aca="false">-Supuestos!$B$15</f>
         <v>-30</v>
       </c>
-      <c r="G11" s="19" t="n">
+      <c r="G11" s="9" t="n">
         <f aca="false">-Supuestos!$B$15</f>
         <v>-30</v>
       </c>
-      <c r="H11" s="19" t="n">
+      <c r="H11" s="9" t="n">
         <f aca="false">-Supuestos!$B$15</f>
         <v>-30</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="B12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="12" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="40" t="s">
+        <v>149</v>
+      </c>
+      <c r="B12" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="13" t="n">
         <f aca="false">SUM(C6,C8:C11)</f>
         <v>-160</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="13" t="n">
         <f aca="false">SUM(D6,D8:D11)</f>
         <v>-160</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <f aca="false">SUM(E6,E8:E11)</f>
         <v>-160</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <f aca="false">SUM(F6,F8:F11)</f>
         <v>-160</v>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="G12" s="13" t="n">
         <f aca="false">SUM(G6,G8:G11)</f>
         <v>-160</v>
       </c>
-      <c r="H12" s="12" t="n">
+      <c r="H12" s="13" t="n">
         <f aca="false">SUM(H6,H8:H11)</f>
         <v>-160</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="B13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="12" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="40" t="s">
+        <v>150</v>
+      </c>
+      <c r="B13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="13" t="n">
         <f aca="false">C7+SUM(C8:C11)</f>
         <v>65</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <f aca="false">D7+SUM(D8:D11)</f>
         <v>65</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <f aca="false">E7+SUM(E8:E11)</f>
         <v>65</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <f aca="false">F7+SUM(F8:F11)</f>
         <v>65</v>
       </c>
-      <c r="G13" s="12" t="n">
+      <c r="G13" s="13" t="n">
         <f aca="false">G7+SUM(G8:G11)</f>
         <v>65</v>
       </c>
-      <c r="H13" s="12" t="n">
+      <c r="H13" s="13" t="n">
         <f aca="false">H7+SUM(H8:H11)</f>
         <v>65</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="19" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="B14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="9" t="n">
         <f aca="false">-MAX(0,C13)*Supuestos!$B$16</f>
         <v>-17.55</v>
       </c>
-      <c r="D14" s="19" t="n">
+      <c r="D14" s="9" t="n">
         <f aca="false">-MAX(0,D13)*Supuestos!$B$16</f>
         <v>-17.55</v>
       </c>
-      <c r="E14" s="19" t="n">
+      <c r="E14" s="9" t="n">
         <f aca="false">-MAX(0,E13)*Supuestos!$B$16</f>
         <v>-17.55</v>
       </c>
-      <c r="F14" s="19" t="n">
+      <c r="F14" s="9" t="n">
         <f aca="false">-MAX(0,F13)*Supuestos!$B$16</f>
         <v>-17.55</v>
       </c>
-      <c r="G14" s="19" t="n">
+      <c r="G14" s="9" t="n">
         <f aca="false">-MAX(0,G13)*Supuestos!$B$16</f>
         <v>-17.55</v>
       </c>
-      <c r="H14" s="19" t="n">
+      <c r="H14" s="9" t="n">
         <f aca="false">-MAX(0,H13)*Supuestos!$B$16</f>
         <v>-17.55</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="12" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="B15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="13" t="n">
         <f aca="false">C13+C14</f>
         <v>47.45</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="13" t="n">
         <f aca="false">D13+D14</f>
         <v>47.45</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="13" t="n">
         <f aca="false">E13+E14</f>
         <v>47.45</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F15" s="13" t="n">
         <f aca="false">F13+F14</f>
         <v>47.45</v>
       </c>
-      <c r="G15" s="12" t="n">
+      <c r="G15" s="13" t="n">
         <f aca="false">G13+G14</f>
         <v>47.45</v>
       </c>
-      <c r="H15" s="12" t="n">
+      <c r="H15" s="13" t="n">
         <f aca="false">H13+H14</f>
         <v>47.45</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B16" s="19" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="B16" s="9" t="n">
         <f aca="false">-Inversion!$B$13</f>
         <v>-88</v>
       </c>
-      <c r="C16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="B17" s="17" t="n">
+      <c r="C16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="41" t="s">
+        <v>154</v>
+      </c>
+      <c r="B17" s="22" t="n">
         <f aca="false">B15+B16</f>
         <v>-88</v>
       </c>
-      <c r="C17" s="17" t="n">
+      <c r="C17" s="22" t="n">
         <f aca="false">C15+C16</f>
         <v>47.45</v>
       </c>
-      <c r="D17" s="17" t="n">
+      <c r="D17" s="22" t="n">
         <f aca="false">D15+D16</f>
         <v>47.45</v>
       </c>
-      <c r="E17" s="17" t="n">
+      <c r="E17" s="22" t="n">
         <f aca="false">E15+E16</f>
         <v>47.45</v>
       </c>
-      <c r="F17" s="17" t="n">
+      <c r="F17" s="22" t="n">
         <f aca="false">F15+F16</f>
         <v>47.45</v>
       </c>
-      <c r="G17" s="17" t="n">
+      <c r="G17" s="22" t="n">
         <f aca="false">G15+G16</f>
         <v>47.45</v>
       </c>
-      <c r="H17" s="17" t="n">
+      <c r="H17" s="22" t="n">
         <f aca="false">H15+H16</f>
         <v>47.45</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="s">
-        <v>81</v>
-      </c>
-      <c r="B18" s="17" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="41" t="s">
+        <v>155</v>
+      </c>
+      <c r="B18" s="22" t="n">
         <f aca="false">B17</f>
         <v>-88</v>
       </c>
-      <c r="C18" s="17" t="n">
+      <c r="C18" s="22" t="n">
         <f aca="false">B18+C17</f>
         <v>-40.55</v>
       </c>
-      <c r="D18" s="17" t="n">
+      <c r="D18" s="22" t="n">
         <f aca="false">C18+D17</f>
         <v>6.90000000000001</v>
       </c>
-      <c r="E18" s="17" t="n">
+      <c r="E18" s="22" t="n">
         <f aca="false">D18+E17</f>
         <v>54.35</v>
       </c>
-      <c r="F18" s="17" t="n">
+      <c r="F18" s="22" t="n">
         <f aca="false">E18+F17</f>
         <v>101.8</v>
       </c>
-      <c r="G18" s="17" t="n">
+      <c r="G18" s="22" t="n">
         <f aca="false">F18+G17</f>
         <v>149.25</v>
       </c>
-      <c r="H18" s="17" t="n">
+      <c r="H18" s="22" t="n">
         <f aca="false">G18+H17</f>
         <v>196.7</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
-        <v>82</v>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -2431,7 +3795,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -2439,247 +3803,247 @@
   <dimension ref="A1:C23"/>
   <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="62"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="A1" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B5" s="19" t="n">
+      <c r="C3" s="4" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="B4" s="42"/>
+      <c r="C4" s="42"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="B5" s="9" t="n">
         <f aca="false">Inversion!$B$13</f>
         <v>88</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B6" s="12" t="n">
+      <c r="C5" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="B6" s="13" t="n">
         <f aca="false">MAX(0,-MIN('Flujo de Caja'!$B$18:$H$18)-Inversion!$B$13)</f>
         <v>0</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="B7" s="17" t="n">
+      <c r="C6" s="3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="40" t="s">
+        <v>165</v>
+      </c>
+      <c r="B7" s="22" t="n">
         <f aca="false">MAX(0,-MIN('Flujo de Caja'!$B$18:$H$18))</f>
         <v>88</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="B8" s="22"/>
-      <c r="C8" s="22"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B9" s="12" t="n">
+      <c r="C7" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B8" s="42"/>
+      <c r="C8" s="42"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="B9" s="13" t="n">
         <f aca="false">NPV(Supuestos!$B$20,'Flujo de Caja'!$C$17:$H$17)+'Flujo de Caja'!$B$17</f>
         <v>187.479126512871</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B10" s="23" t="n">
+      <c r="C9" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="B10" s="43" t="n">
         <f aca="false">IFERROR(IRR('Flujo de Caja'!$B$17:$H$17,0.02),"No calculable")</f>
         <v>0.489910783440648</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B11" s="23" t="n">
+      <c r="C10" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B11" s="43" t="n">
         <f aca="false">IFERROR((1+B10)^12-1,"No calculable")</f>
         <v>118.652881325872</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B12" s="24" t="n">
+      <c r="C11" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="B12" s="44" t="n">
         <f aca="false">Supuestos!$B$17</f>
         <v>0.12</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="B13" s="11" t="n">
+      <c r="C12" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="B13" s="12" t="n">
         <f aca="false" t="array" ref="B13:B13">IF(INDEX('Flujo de Caja'!$B$18:$H$18,1,COLUMNS('Flujo de Caja'!$B$18:$H$18))&lt;0,"No recupera en 6 meses",COUNTIF('Flujo de Caja'!$B$18:$H$18,"&lt;0"))</f>
         <v>2</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="B14" s="12" t="n">
+      <c r="C13" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="B14" s="13" t="n">
         <f aca="false" t="array" ref="B14:B14">INDEX('Flujo de Caja'!$B$18:$H$18,1,COLUMNS('Flujo de Caja'!$B$18:$H$18))</f>
         <v>196.7</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="B15" s="23" t="n">
+      <c r="C14" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="B15" s="43" t="n">
         <f aca="false">IFERROR(B14/B7,0)</f>
         <v>2.23522727272727</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="B17" s="11" t="n">
+      <c r="C15" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="B16" s="42"/>
+      <c r="C16" s="42"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="B17" s="12" t="n">
         <f aca="false">ROUNDUP(Supuestos!$B$23/Supuestos!$B$24,0)</f>
         <v>11</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B18" s="18" t="n">
+      <c r="C17" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B18" s="39" t="n">
         <f aca="false">Supuestos!$B$21</f>
         <v>15</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="B19" s="19" t="n">
+      <c r="C18" s="3" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="B19" s="9" t="n">
         <f aca="false">B17*Supuestos!$B$4</f>
         <v>165</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="B20" s="19" t="n">
+      <c r="C19" s="3" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B20" s="9" t="n">
         <f aca="false">B18*Supuestos!$B$24-Supuestos!$B$23</f>
         <v>65</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="B21" s="23" t="n">
+      <c r="C20" s="3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="B21" s="43" t="n">
         <f aca="false">IFERROR(B20/(B18*Supuestos!$B$4),0)</f>
         <v>0.288888888888889</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
+      <c r="C21" s="3" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="B22" s="42"/>
+      <c r="C22" s="42"/>
     </row>
     <row r="23" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="B23" s="25" t="str">
+      <c r="A23" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B23" s="45" t="str">
         <f aca="false">IF(AND(ISNUMBER(B9),B9&gt;0,B18&gt;=B17),"VIABLE: VAN positivo y la capacidad supera el punto de equilibrio",IF(B18&lt;B17,"NO VIABLE: la capacidad no alcanza el punto de equilibrio","NO VIABLE en 6 meses: VAN negativo"))</f>
         <v>VIABLE: VAN positivo y la capacidad supera el punto de equilibrio</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>121</v>
+      <c r="C23" s="3" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -2696,7 +4060,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -2704,596 +4068,596 @@
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="2" style="1" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
+      <c r="A1" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="26"/>
-      <c r="O2" s="26"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
-        <v>124</v>
-      </c>
-      <c r="B4" s="17" t="n">
+      <c r="A2" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="40" t="s">
+        <v>198</v>
+      </c>
+      <c r="B4" s="22" t="n">
         <f aca="false">F14</f>
         <v>1048</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
-        <v>125</v>
-      </c>
-      <c r="B5" s="27" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="40" t="s">
+        <v>199</v>
+      </c>
+      <c r="B5" s="46" t="n">
         <f aca="false">COUNT(D9:D14)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="N8" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="O8" s="3" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="28" t="n">
+      <c r="A8" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="B9" s="23" t="n">
+      <c r="B9" s="43" t="n">
         <f aca="false">F9/$B$4</f>
         <v>0.236641221374046</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="19" t="n">
+      <c r="C9" s="8"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="9" t="n">
         <f aca="false">-'Flujo de Caja'!C12+Inversion!$B$13</f>
         <v>248</v>
       </c>
-      <c r="F9" s="12" t="n">
+      <c r="F9" s="13" t="n">
         <f aca="false">SUM($E$9:E9)</f>
         <v>248</v>
       </c>
-      <c r="G9" s="12" t="str">
+      <c r="G9" s="13" t="str">
         <f aca="false">IF(D9="","",C9*$B$4)</f>
         <v/>
       </c>
-      <c r="H9" s="12" t="str">
+      <c r="H9" s="13" t="str">
         <f aca="false">IF(D9="","",G9-D9)</f>
         <v/>
       </c>
-      <c r="I9" s="12" t="str">
+      <c r="I9" s="13" t="str">
         <f aca="false">IF(D9="","",G9-F9)</f>
         <v/>
       </c>
-      <c r="J9" s="29" t="str">
+      <c r="J9" s="49" t="str">
         <f aca="false">IF(D9="","",IFERROR(G9/D9,0))</f>
         <v/>
       </c>
-      <c r="K9" s="29" t="str">
+      <c r="K9" s="49" t="str">
         <f aca="false">IF(D9="","",IFERROR(G9/F9,0))</f>
         <v/>
       </c>
-      <c r="L9" s="12" t="str">
+      <c r="L9" s="13" t="str">
         <f aca="false">IF(D9="","",IFERROR($B$4/J9,0))</f>
         <v/>
       </c>
-      <c r="M9" s="12" t="str">
+      <c r="M9" s="13" t="str">
         <f aca="false">IF(D9="","",L9-D9)</f>
         <v/>
       </c>
-      <c r="N9" s="12" t="str">
+      <c r="N9" s="13" t="str">
         <f aca="false">IF(D9="","",$B$4-L9)</f>
         <v/>
       </c>
-      <c r="O9" s="29" t="str">
+      <c r="O9" s="49" t="str">
         <f aca="false">IF(D9="","",IFERROR(($B$4-G9)/($B$4-D9),0))</f>
         <v/>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="47" t="n">
         <v>2</v>
       </c>
-      <c r="B10" s="23" t="n">
+      <c r="B10" s="43" t="n">
         <f aca="false">F10/$B$4</f>
         <v>0.389312977099237</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="19" t="n">
+      <c r="C10" s="8"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="9" t="n">
         <f aca="false">-'Flujo de Caja'!D12</f>
         <v>160</v>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="13" t="n">
         <f aca="false">SUM($E$9:E10)</f>
         <v>408</v>
       </c>
-      <c r="G10" s="12" t="str">
+      <c r="G10" s="13" t="str">
         <f aca="false">IF(D10="","",C10*$B$4)</f>
         <v/>
       </c>
-      <c r="H10" s="12" t="str">
+      <c r="H10" s="13" t="str">
         <f aca="false">IF(D10="","",G10-D10)</f>
         <v/>
       </c>
-      <c r="I10" s="12" t="str">
+      <c r="I10" s="13" t="str">
         <f aca="false">IF(D10="","",G10-F10)</f>
         <v/>
       </c>
-      <c r="J10" s="29" t="str">
+      <c r="J10" s="49" t="str">
         <f aca="false">IF(D10="","",IFERROR(G10/D10,0))</f>
         <v/>
       </c>
-      <c r="K10" s="29" t="str">
+      <c r="K10" s="49" t="str">
         <f aca="false">IF(D10="","",IFERROR(G10/F10,0))</f>
         <v/>
       </c>
-      <c r="L10" s="12" t="str">
+      <c r="L10" s="13" t="str">
         <f aca="false">IF(D10="","",IFERROR($B$4/J10,0))</f>
         <v/>
       </c>
-      <c r="M10" s="12" t="str">
+      <c r="M10" s="13" t="str">
         <f aca="false">IF(D10="","",L10-D10)</f>
         <v/>
       </c>
-      <c r="N10" s="12" t="str">
+      <c r="N10" s="13" t="str">
         <f aca="false">IF(D10="","",$B$4-L10)</f>
         <v/>
       </c>
-      <c r="O10" s="29" t="str">
+      <c r="O10" s="49" t="str">
         <f aca="false">IF(D10="","",IFERROR(($B$4-G10)/($B$4-D10),0))</f>
         <v/>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="47" t="n">
         <v>3</v>
       </c>
-      <c r="B11" s="23" t="n">
+      <c r="B11" s="43" t="n">
         <f aca="false">F11/$B$4</f>
         <v>0.541984732824428</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="19" t="n">
+      <c r="C11" s="8"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="9" t="n">
         <f aca="false">-'Flujo de Caja'!E12</f>
         <v>160</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <f aca="false">SUM($E$9:E11)</f>
         <v>568</v>
       </c>
-      <c r="G11" s="12" t="str">
+      <c r="G11" s="13" t="str">
         <f aca="false">IF(D11="","",C11*$B$4)</f>
         <v/>
       </c>
-      <c r="H11" s="12" t="str">
+      <c r="H11" s="13" t="str">
         <f aca="false">IF(D11="","",G11-D11)</f>
         <v/>
       </c>
-      <c r="I11" s="12" t="str">
+      <c r="I11" s="13" t="str">
         <f aca="false">IF(D11="","",G11-F11)</f>
         <v/>
       </c>
-      <c r="J11" s="29" t="str">
+      <c r="J11" s="49" t="str">
         <f aca="false">IF(D11="","",IFERROR(G11/D11,0))</f>
         <v/>
       </c>
-      <c r="K11" s="29" t="str">
+      <c r="K11" s="49" t="str">
         <f aca="false">IF(D11="","",IFERROR(G11/F11,0))</f>
         <v/>
       </c>
-      <c r="L11" s="12" t="str">
+      <c r="L11" s="13" t="str">
         <f aca="false">IF(D11="","",IFERROR($B$4/J11,0))</f>
         <v/>
       </c>
-      <c r="M11" s="12" t="str">
+      <c r="M11" s="13" t="str">
         <f aca="false">IF(D11="","",L11-D11)</f>
         <v/>
       </c>
-      <c r="N11" s="12" t="str">
+      <c r="N11" s="13" t="str">
         <f aca="false">IF(D11="","",$B$4-L11)</f>
         <v/>
       </c>
-      <c r="O11" s="29" t="str">
+      <c r="O11" s="49" t="str">
         <f aca="false">IF(D11="","",IFERROR(($B$4-G11)/($B$4-D11),0))</f>
         <v/>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="28" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="47" t="n">
         <v>4</v>
       </c>
-      <c r="B12" s="23" t="n">
+      <c r="B12" s="43" t="n">
         <f aca="false">F12/$B$4</f>
         <v>0.694656488549618</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="19" t="n">
+      <c r="C12" s="8"/>
+      <c r="D12" s="48"/>
+      <c r="E12" s="9" t="n">
         <f aca="false">-'Flujo de Caja'!F12</f>
         <v>160</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <f aca="false">SUM($E$9:E12)</f>
         <v>728</v>
       </c>
-      <c r="G12" s="12" t="str">
+      <c r="G12" s="13" t="str">
         <f aca="false">IF(D12="","",C12*$B$4)</f>
         <v/>
       </c>
-      <c r="H12" s="12" t="str">
+      <c r="H12" s="13" t="str">
         <f aca="false">IF(D12="","",G12-D12)</f>
         <v/>
       </c>
-      <c r="I12" s="12" t="str">
+      <c r="I12" s="13" t="str">
         <f aca="false">IF(D12="","",G12-F12)</f>
         <v/>
       </c>
-      <c r="J12" s="29" t="str">
+      <c r="J12" s="49" t="str">
         <f aca="false">IF(D12="","",IFERROR(G12/D12,0))</f>
         <v/>
       </c>
-      <c r="K12" s="29" t="str">
+      <c r="K12" s="49" t="str">
         <f aca="false">IF(D12="","",IFERROR(G12/F12,0))</f>
         <v/>
       </c>
-      <c r="L12" s="12" t="str">
+      <c r="L12" s="13" t="str">
         <f aca="false">IF(D12="","",IFERROR($B$4/J12,0))</f>
         <v/>
       </c>
-      <c r="M12" s="12" t="str">
+      <c r="M12" s="13" t="str">
         <f aca="false">IF(D12="","",L12-D12)</f>
         <v/>
       </c>
-      <c r="N12" s="12" t="str">
+      <c r="N12" s="13" t="str">
         <f aca="false">IF(D12="","",$B$4-L12)</f>
         <v/>
       </c>
-      <c r="O12" s="29" t="str">
+      <c r="O12" s="49" t="str">
         <f aca="false">IF(D12="","",IFERROR(($B$4-G12)/($B$4-D12),0))</f>
         <v/>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="28" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="47" t="n">
         <v>5</v>
       </c>
-      <c r="B13" s="23" t="n">
+      <c r="B13" s="43" t="n">
         <f aca="false">F13/$B$4</f>
         <v>0.847328244274809</v>
       </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="19" t="n">
+      <c r="C13" s="8"/>
+      <c r="D13" s="48"/>
+      <c r="E13" s="9" t="n">
         <f aca="false">-'Flujo de Caja'!G12</f>
         <v>160</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <f aca="false">SUM($E$9:E13)</f>
         <v>888</v>
       </c>
-      <c r="G13" s="12" t="str">
+      <c r="G13" s="13" t="str">
         <f aca="false">IF(D13="","",C13*$B$4)</f>
         <v/>
       </c>
-      <c r="H13" s="12" t="str">
+      <c r="H13" s="13" t="str">
         <f aca="false">IF(D13="","",G13-D13)</f>
         <v/>
       </c>
-      <c r="I13" s="12" t="str">
+      <c r="I13" s="13" t="str">
         <f aca="false">IF(D13="","",G13-F13)</f>
         <v/>
       </c>
-      <c r="J13" s="29" t="str">
+      <c r="J13" s="49" t="str">
         <f aca="false">IF(D13="","",IFERROR(G13/D13,0))</f>
         <v/>
       </c>
-      <c r="K13" s="29" t="str">
+      <c r="K13" s="49" t="str">
         <f aca="false">IF(D13="","",IFERROR(G13/F13,0))</f>
         <v/>
       </c>
-      <c r="L13" s="12" t="str">
+      <c r="L13" s="13" t="str">
         <f aca="false">IF(D13="","",IFERROR($B$4/J13,0))</f>
         <v/>
       </c>
-      <c r="M13" s="12" t="str">
+      <c r="M13" s="13" t="str">
         <f aca="false">IF(D13="","",L13-D13)</f>
         <v/>
       </c>
-      <c r="N13" s="12" t="str">
+      <c r="N13" s="13" t="str">
         <f aca="false">IF(D13="","",$B$4-L13)</f>
         <v/>
       </c>
-      <c r="O13" s="29" t="str">
+      <c r="O13" s="49" t="str">
         <f aca="false">IF(D13="","",IFERROR(($B$4-G13)/($B$4-D13),0))</f>
         <v/>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="28" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="47" t="n">
         <v>6</v>
       </c>
-      <c r="B14" s="23" t="n">
+      <c r="B14" s="43" t="n">
         <f aca="false">F14/$B$4</f>
         <v>1</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="19" t="n">
+      <c r="C14" s="8"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="9" t="n">
         <f aca="false">-'Flujo de Caja'!H12</f>
         <v>160</v>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="13" t="n">
         <f aca="false">SUM($E$9:E14)</f>
         <v>1048</v>
       </c>
-      <c r="G14" s="12" t="str">
+      <c r="G14" s="13" t="str">
         <f aca="false">IF(D14="","",C14*$B$4)</f>
         <v/>
       </c>
-      <c r="H14" s="12" t="str">
+      <c r="H14" s="13" t="str">
         <f aca="false">IF(D14="","",G14-D14)</f>
         <v/>
       </c>
-      <c r="I14" s="12" t="str">
+      <c r="I14" s="13" t="str">
         <f aca="false">IF(D14="","",G14-F14)</f>
         <v/>
       </c>
-      <c r="J14" s="29" t="str">
+      <c r="J14" s="49" t="str">
         <f aca="false">IF(D14="","",IFERROR(G14/D14,0))</f>
         <v/>
       </c>
-      <c r="K14" s="29" t="str">
+      <c r="K14" s="49" t="str">
         <f aca="false">IF(D14="","",IFERROR(G14/F14,0))</f>
         <v/>
       </c>
-      <c r="L14" s="12" t="str">
+      <c r="L14" s="13" t="str">
         <f aca="false">IF(D14="","",IFERROR($B$4/J14,0))</f>
         <v/>
       </c>
-      <c r="M14" s="12" t="str">
+      <c r="M14" s="13" t="str">
         <f aca="false">IF(D14="","",L14-D14)</f>
         <v/>
       </c>
-      <c r="N14" s="12" t="str">
+      <c r="N14" s="13" t="str">
         <f aca="false">IF(D14="","",$B$4-L14)</f>
         <v/>
       </c>
-      <c r="O14" s="29" t="str">
+      <c r="O14" s="49" t="str">
         <f aca="false">IF(D14="","",IFERROR(($B$4-G14)/($B$4-D14),0))</f>
         <v/>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="B17" s="12" t="str">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="B16" s="42"/>
+      <c r="C16" s="42"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="B17" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(F9:F14,$B$5))</f>
         <v>Sin datos</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="B18" s="12" t="str">
+      <c r="C17" s="3" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="B18" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(G9:G14,$B$5))</f>
         <v>Sin datos</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="B19" s="12" t="str">
+      <c r="C18" s="3" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="B19" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(D9:D14,$B$5))</f>
         <v>Sin datos</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="B20" s="12" t="str">
+      <c r="C19" s="3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="B20" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(H9:H14,$B$5))</f>
         <v>Sin datos</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="B21" s="12" t="str">
+      <c r="C20" s="3" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="B21" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(I9:I14,$B$5))</f>
         <v>Sin datos</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="B22" s="29" t="str">
+      <c r="C21" s="3" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="B22" s="49" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(J9:J14,$B$5))</f>
         <v>Sin datos</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="B23" s="29" t="str">
+      <c r="C22" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="B23" s="49" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(K9:K14,$B$5))</f>
         <v>Sin datos</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="B24" s="12" t="str">
+      <c r="C23" s="3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="B24" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(L9:L14,$B$5))</f>
         <v>Sin datos</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="B25" s="12" t="str">
+      <c r="C24" s="3" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="B25" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(M9:M14,$B$5))</f>
         <v>Sin datos</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="B26" s="12" t="str">
+      <c r="C25" s="3" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="B26" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(N9:N14,$B$5))</f>
         <v>Sin datos</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="B27" s="29" t="str">
+      <c r="C26" s="3" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="B27" s="49" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(O9:O14,$B$5))</f>
         <v>Sin datos</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14" t="s">
-        <v>163</v>
-      </c>
-      <c r="B28" s="20" t="str">
+      <c r="C27" s="3" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="19" t="s">
+        <v>237</v>
+      </c>
+      <c r="B28" s="40" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",IF(B22&gt;=1,"Bajo presupuesto","Sobre presupuesto"))</f>
         <v>Sin datos</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="B29" s="20" t="str">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="19" t="s">
+        <v>238</v>
+      </c>
+      <c r="B29" s="40" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",IF(B23&gt;=1,"Adelantado / a tiempo","Atrasado"))</f>
         <v>Sin datos</v>
       </c>

</xml_diff>

<commit_message>
Separar costos y gastos mensuales en dos tablas
La hoja Gastos Mensuales pasa a Costos y Gastos: tabla de costos (producir
las clases), tabla de gastos (vender y administrar), margen del servicio y
utilidad mensual. Se mantienen los vinculos con Supuestos y Gastos Inicio.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FyrtynBGssxjxAFxFhXjrS
</commit_message>
<xml_diff>
--- a/Viabilidad_Academia_LoL.xlsx
+++ b/Viabilidad_Academia_LoL.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Supuestos" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Inversion" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Gastos Inicio" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Gastos Mensuales" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Costos y Gastos" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Flujo de Caja" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Indicadores" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Valor Ganado" sheetId="7" state="visible" r:id="rId9"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="254">
   <si>
     <t xml:space="preserve">Academia de League of Legends - Supuestos del modelo</t>
   </si>
@@ -97,19 +97,19 @@
     <t xml:space="preserve">Plataforma y software mensual (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Viene de la hoja Gastos Mensuales (categoria Plataforma, solo lo incluido)</t>
+    <t xml:space="preserve">Viene de la hoja Costos y Gastos (categoria Plataforma, solo lo incluido)</t>
   </si>
   <si>
     <t xml:space="preserve">Marketing mensual (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Viene de la hoja Gastos Mensuales (categoria Marketing, solo lo incluido)</t>
+    <t xml:space="preserve">Viene de la hoja Costos y Gastos (categoria Marketing, solo lo incluido)</t>
   </si>
   <si>
     <t xml:space="preserve">Otros gastos mensuales (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Viene de la hoja Gastos Mensuales (categoria Otros, solo lo incluido)</t>
+    <t xml:space="preserve">Viene de la hoja Costos y Gastos (categoria Otros, solo lo incluido)</t>
   </si>
   <si>
     <t xml:space="preserve">Tasa de impuesto sobre utilidad</t>
@@ -310,10 +310,10 @@
     <t xml:space="preserve">Viene de la hoja Inversion</t>
   </si>
   <si>
-    <t xml:space="preserve">Gasto mensual total (coaches + gastos incluidos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Viene de la hoja Gastos Mensuales</t>
+    <t xml:space="preserve">Costos + gastos mensuales (incluidos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viene de la hoja Costos y Gastos</t>
   </si>
   <si>
     <t xml:space="preserve">Meses de gastos como reserva</t>
@@ -334,22 +334,31 @@
     <t xml:space="preserve">Inversion inicial + fondo de reserva</t>
   </si>
   <si>
-    <t xml:space="preserve">Gastos mensuales - en que invertir cada mes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cada gasto tiene categoria (alimenta la hoja Supuestos) y prioridad. Solo lo marcado 'Si' entra al flujo de caja. Los sueldos de coaches se calculan en Supuestos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gasto mensual</t>
+    <t xml:space="preserve">Costos y gastos mensuales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COSTO = lo que pagas para producir las clases (sin esto no hay servicio). GASTO = lo que pagas para vender y administrar el negocio. Solo lo marcado 'Si' entra al flujo de caja. Edita las celdas amarillas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. COSTOS - producir las clases</t>
   </si>
   <si>
     <t xml:space="preserve">Categoria</t>
   </si>
   <si>
-    <t xml:space="preserve">Costo mensual (USD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Discord Nitro / boost del servidor</t>
+    <t xml:space="preserve">Monto mensual (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sueldos de coaches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sueldos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viene de Supuestos: (coaches - no cobran) x sueldo x horas. Se edita alli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discord Nitro / boost del servidor (aula de clases)</t>
   </si>
   <si>
     <t xml:space="preserve">Plataforma</t>
@@ -361,70 +370,106 @@
     <t xml:space="preserve">Herramienta de analisis de partidas / VOD</t>
   </si>
   <si>
+    <t xml:space="preserve">TOTAL COSTOS MENSUALES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. GASTOS - vender y administrar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anuncios en redes (TikTok / Instagram)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dato del usuario: marketing = 80 USD/mes (repartido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colaboraciones con streamers / creadores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Premios torneos internos (RP / skins)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: retencion de alumnos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internet y servicios (proporcion)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Otros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dato del usuario: otros = 30 USD/mes (repartido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Administracion y contabilidad</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dominio y hosting web</t>
   </si>
   <si>
     <t xml:space="preserve">Supuesto: solo si hay pagina web</t>
   </si>
   <si>
-    <t xml:space="preserve">Anuncios en redes (TikTok / Instagram)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marketing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dato del usuario: marketing = 80 USD/mes (repartido)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Colaboraciones con streamers / creadores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Premios torneos internos (RP / skins)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supuesto: retencion de alumnos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Internet y servicios (proporcion)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Otros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dato del usuario: otros = 30 USD/mes (repartido)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Administracion y contabilidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL GASTOS (sin sueldos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resumen mensual (incluido)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USD / mes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sueldos de coaches</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Viene de Supuestos (coaches que cobran x sueldo x horas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GASTO MENSUAL TOTAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Por prioridad (incluido)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingreso mensual esperado (mes 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingreso - gasto mensual total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Si es negativo, recorta primero lo Opcional y luego lo Importante</t>
+    <t xml:space="preserve">TOTAL GASTOS MENSUALES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. RESULTADO MENSUAL (mes 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingreso mensual esperado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viene de Flujo de Caja (alumnos x precio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(-) Costos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabla 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARGEN DEL SERVICIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si es negativo, dar clases no es rentable: sube precio o alumnos por coach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Margen del servicio (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Margen / ingreso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(-) Gastos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabla 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UTILIDAD MENSUAL (antes de impuestos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si es negativa, recorta gastos Opcionales y luego Importantes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. RESUMEN PARA EL MODELO (solo lo incluido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alimenta la hoja Supuestos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COSTOS + GASTOS MENSUALES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control (debe ser 0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si no es 0, hay una fila con categoria vacia o mal escrita</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. POR PRIORIDAD (costos + gastos incluidos)</t>
   </si>
   <si>
     <t xml:space="preserve">Flujo de caja proyectado - 6 meses (USD)</t>
@@ -749,18 +794,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="166" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="167" formatCode="0.0%;\(0.0%\);\-"/>
     <numFmt numFmtId="168" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="169" formatCode="0.000%"/>
-    <numFmt numFmtId="170" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
-    <numFmt numFmtId="171" formatCode="0"/>
-    <numFmt numFmtId="172" formatCode="0.00"/>
+    <numFmt numFmtId="170" formatCode="0"/>
+    <numFmt numFmtId="171" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
+    <numFmt numFmtId="172" formatCode="0.0%;\(0.0%\);\-"/>
+    <numFmt numFmtId="173" formatCode="0.00"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -836,6 +882,14 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="18"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -855,7 +909,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -871,7 +925,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3864"/>
-        <bgColor rgb="FF333399"/>
+        <bgColor rgb="FF2F5597"/>
       </patternFill>
     </fill>
     <fill>
@@ -884,6 +938,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
         <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF833C0B"/>
+        <bgColor rgb="FF993366"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F5597"/>
+        <bgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
   </fills>
@@ -936,7 +1002,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="55">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -997,19 +1063,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1021,10 +1079,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="168" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1033,23 +1087,71 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1057,31 +1159,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1089,6 +1183,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1097,18 +1195,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1125,15 +1215,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1146,7 +1232,28 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="6">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFE699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1223,9 +1330,9 @@
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF833C0B"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF2F5597"/>
       <rgbColor rgb="FF555555"/>
     </indexedColors>
   </colors>
@@ -1267,8 +1374,8 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.221634162256217"/>
-          <c:y val="0.0311366762535951"/>
+          <c:x val="0.221678448432119"/>
+          <c:y val="0.0312656328164082"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -1399,11 +1506,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="14966397"/>
-        <c:axId val="97645602"/>
+        <c:axId val="26743232"/>
+        <c:axId val="89650305"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="14966397"/>
+        <c:axId val="26743232"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1469,7 +1576,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97645602"/>
+        <c:crossAx val="89650305"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1477,7 +1584,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="97645602"/>
+        <c:axId val="89650305"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1553,7 +1660,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14966397"/>
+        <c:crossAx val="26743232"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1592,9 +1699,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>135720</xdr:colOff>
+      <xdr:colOff>135360</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>145080</xdr:rowOff>
+      <xdr:rowOff>144720</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1603,7 +1710,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="1380960" y="3667320"/>
-        <a:ext cx="9930600" cy="2878560"/>
+        <a:ext cx="9930240" cy="2878200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1931,7 +2038,7 @@
         <v>22</v>
       </c>
       <c r="B13" s="9" t="n">
-        <f aca="false">'Gastos Mensuales'!$F$21</f>
+        <f aca="false">'Costos y Gastos'!$F$38</f>
         <v>10</v>
       </c>
       <c r="C13" s="3" t="s">
@@ -1943,7 +2050,7 @@
         <v>24</v>
       </c>
       <c r="B14" s="9" t="n">
-        <f aca="false">'Gastos Mensuales'!$F$22</f>
+        <f aca="false">'Costos y Gastos'!$F$39</f>
         <v>80</v>
       </c>
       <c r="C14" s="3" t="s">
@@ -1955,7 +2062,7 @@
         <v>26</v>
       </c>
       <c r="B15" s="9" t="n">
-        <f aca="false">'Gastos Mensuales'!$F$23</f>
+        <f aca="false">'Costos y Gastos'!$F$40</f>
         <v>30</v>
       </c>
       <c r="C15" s="3" t="s">
@@ -2103,7 +2210,7 @@
       <c r="A4" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="15" t="n">
+      <c r="B4" s="9" t="n">
         <f aca="false">'Gastos Inicio'!$E$23</f>
         <v>80</v>
       </c>
@@ -2115,7 +2222,7 @@
       <c r="A5" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="15" t="n">
+      <c r="B5" s="9" t="n">
         <f aca="false">'Gastos Inicio'!$E$24</f>
         <v>0</v>
       </c>
@@ -2127,7 +2234,7 @@
       <c r="A6" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B6" s="15" t="n">
+      <c r="B6" s="9" t="n">
         <f aca="false">'Gastos Inicio'!$E$25</f>
         <v>0</v>
       </c>
@@ -2136,31 +2243,31 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="18"/>
+      <c r="A7" s="15"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="18"/>
+      <c r="A8" s="15"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16"/>
-      <c r="B9" s="17"/>
-      <c r="C9" s="18"/>
+      <c r="A9" s="15"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="20" t="n">
+      <c r="B10" s="18" t="n">
         <f aca="false">SUM(B4:B9)</f>
         <v>80</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="15" t="s">
         <v>53</v>
       </c>
       <c r="B11" s="8" t="n">
@@ -2171,7 +2278,7 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="15" t="s">
         <v>55</v>
       </c>
       <c r="B12" s="13" t="n">
@@ -2180,10 +2287,10 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="22" t="n">
+      <c r="B13" s="19" t="n">
         <f aca="false">B10+B12</f>
         <v>88</v>
       </c>
@@ -2210,12 +2317,12 @@
   <dimension ref="A1:F32"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="62"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2229,14 +2336,14 @@
       <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
@@ -2258,403 +2365,403 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="26" t="n">
+      <c r="C5" s="23" t="n">
         <v>50</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="E5" s="27" t="n">
+      <c r="E5" s="13" t="n">
         <f aca="false">IF(D5="Si",N(C5),0)</f>
         <v>50</v>
       </c>
-      <c r="F5" s="28" t="s">
+      <c r="F5" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="C6" s="26" t="n">
+      <c r="C6" s="23" t="n">
         <v>30</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="D6" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="13" t="n">
         <f aca="false">IF(D6="Si",N(C6),0)</f>
         <v>30</v>
       </c>
-      <c r="F6" s="28" t="s">
+      <c r="F6" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="C7" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="25" t="s">
+      <c r="C7" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="13" t="n">
         <f aca="false">IF(D7="Si",N(C7),0)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="28" t="s">
+      <c r="F7" s="3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="24" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="C8" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="25" t="s">
+      <c r="C8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="13" t="n">
         <f aca="false">IF(D8="Si",N(C8),0)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="28" t="s">
+      <c r="F8" s="3" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="24" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="C9" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="25" t="s">
+      <c r="C9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="13" t="n">
         <f aca="false">IF(D9="Si",N(C9),0)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="28" t="s">
+      <c r="F9" s="3" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="24" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="C10" s="26" t="n">
+      <c r="C10" s="23" t="n">
         <v>100</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="D10" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="13" t="n">
         <f aca="false">IF(D10="Si",N(C10),0)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="28" t="s">
+      <c r="F10" s="3" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="C11" s="26" t="n">
+      <c r="C11" s="23" t="n">
         <v>300</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="D11" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="E11" s="27" t="n">
+      <c r="E11" s="13" t="n">
         <f aca="false">IF(D11="Si",N(C11),0)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="28" t="s">
+      <c r="F11" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="C12" s="26" t="n">
+      <c r="C12" s="23" t="n">
         <v>50</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="D12" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="E12" s="27" t="n">
+      <c r="E12" s="13" t="n">
         <f aca="false">IF(D12="Si",N(C12),0)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="28" t="s">
+      <c r="F12" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="C13" s="26" t="n">
+      <c r="C13" s="23" t="n">
         <v>150</v>
       </c>
-      <c r="D13" s="25" t="s">
+      <c r="D13" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="E13" s="27" t="n">
+      <c r="E13" s="13" t="n">
         <f aca="false">IF(D13="Si",N(C13),0)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="28" t="s">
+      <c r="F13" s="3" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="24" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="C14" s="26" t="n">
+      <c r="C14" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="D14" s="25" t="s">
+      <c r="D14" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="E14" s="27" t="n">
+      <c r="E14" s="13" t="n">
         <f aca="false">IF(D14="Si",N(C14),0)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="28" t="s">
+      <c r="F14" s="3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="24"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="27" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="13" t="n">
         <f aca="false">IF(D15="Si",N(C15),0)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="28"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="24"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="27" t="n">
+      <c r="F15" s="3"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="13" t="n">
         <f aca="false">IF(D16="Si",N(C16),0)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="28"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="24"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="27" t="n">
+      <c r="F16" s="3"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="13" t="n">
         <f aca="false">IF(D17="Si",N(C17),0)</f>
         <v>0</v>
       </c>
-      <c r="F17" s="28"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="24"/>
-      <c r="B18" s="25"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="27" t="n">
+      <c r="F17" s="3"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="13" t="n">
         <f aca="false">IF(D18="Si",N(C18),0)</f>
         <v>0</v>
       </c>
-      <c r="F18" s="28"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="24"/>
-      <c r="B19" s="25"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="27" t="n">
+      <c r="F18" s="3"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="13" t="n">
         <f aca="false">IF(D19="Si",N(C19),0)</f>
         <v>0</v>
       </c>
-      <c r="F19" s="28"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="29" t="s">
+      <c r="F19" s="3"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C20" s="30" t="n">
+      <c r="C20" s="19" t="n">
         <f aca="false">SUM(C5:C19)</f>
         <v>700</v>
       </c>
-      <c r="E20" s="30" t="n">
+      <c r="E20" s="19" t="n">
         <f aca="false">SUM(E5:E19)</f>
         <v>80</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="31" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="B22" s="31"/>
-      <c r="C22" s="31" t="s">
+      <c r="B22" s="24"/>
+      <c r="C22" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="D22" s="31"/>
-      <c r="E22" s="31" t="s">
+      <c r="D22" s="24"/>
+      <c r="E22" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="F22" s="31"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="32" t="s">
+      <c r="F22" s="24"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="27" t="n">
+      <c r="C23" s="13" t="n">
         <f aca="false">SUMIFS($C$5:$C$19,$B$5:$B$19,"Vital")</f>
         <v>80</v>
       </c>
-      <c r="E23" s="27" t="n">
+      <c r="E23" s="13" t="n">
         <f aca="false">SUMIFS($E$5:$E$19,$B$5:$B$19,"Vital")</f>
         <v>80</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="32" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="C24" s="27" t="n">
+      <c r="C24" s="13" t="n">
         <f aca="false">SUMIFS($C$5:$C$19,$B$5:$B$19,"Importante")</f>
         <v>400</v>
       </c>
-      <c r="E24" s="27" t="n">
+      <c r="E24" s="13" t="n">
         <f aca="false">SUMIFS($E$5:$E$19,$B$5:$B$19,"Importante")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="32" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C25" s="27" t="n">
+      <c r="C25" s="13" t="n">
         <f aca="false">SUMIFS($C$5:$C$19,$B$5:$B$19,"Opcional")</f>
         <v>220</v>
       </c>
-      <c r="E25" s="27" t="n">
+      <c r="E25" s="13" t="n">
         <f aca="false">SUMIFS($E$5:$E$19,$B$5:$B$19,"Opcional")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="33" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B27" s="34"/>
-      <c r="C27" s="34"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="34"/>
-      <c r="F27" s="34"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="32" t="s">
+      <c r="B27" s="25"/>
+      <c r="C27" s="25"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="C28" s="35" t="n">
+      <c r="C28" s="9" t="n">
         <f aca="false">Inversion!$B$13</f>
         <v>88</v>
       </c>
-      <c r="D28" s="28" t="s">
+      <c r="D28" s="3" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="32" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C29" s="35" t="n">
-        <f aca="false">'Gastos Mensuales'!$F$25</f>
+      <c r="C29" s="9" t="n">
+        <f aca="false">'Costos y Gastos'!$F$42</f>
         <v>160</v>
       </c>
-      <c r="D29" s="28" t="s">
+      <c r="D29" s="3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="32" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="C30" s="36" t="n">
+      <c r="C30" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="D30" s="28" t="s">
+      <c r="D30" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="32" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="C31" s="27" t="n">
+      <c r="C31" s="13" t="n">
         <f aca="false">C29*C30</f>
         <v>160</v>
       </c>
-      <c r="D31" s="28" t="s">
+      <c r="D31" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="37" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="27" t="s">
         <v>100</v>
       </c>
-      <c r="C32" s="30" t="n">
+      <c r="C32" s="19" t="n">
         <f aca="false">C28+C31</f>
         <v>248</v>
       </c>
-      <c r="D32" s="28" t="s">
+      <c r="D32" s="3" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2732,447 +2839,642 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="62"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="28" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-    </row>
-    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+    </row>
+    <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="31" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B6" s="32" t="s">
         <v>108</v>
       </c>
-      <c r="C5" s="25" t="s">
-        <v>74</v>
-      </c>
-      <c r="D5" s="26" t="n">
-        <v>10</v>
-      </c>
-      <c r="E5" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F5" s="27" t="n">
-        <f aca="false">IF(E5="Si",N(D5),0)</f>
-        <v>10</v>
-      </c>
-      <c r="G5" s="28" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
-        <v>110</v>
-      </c>
-      <c r="B6" s="25" t="s">
-        <v>108</v>
-      </c>
-      <c r="C6" s="25" t="s">
-        <v>82</v>
-      </c>
-      <c r="D6" s="26" t="n">
-        <v>15</v>
-      </c>
-      <c r="E6" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="F6" s="27" t="n">
-        <f aca="false">IF(E6="Si",N(D6),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G6" s="28" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
-        <v>111</v>
-      </c>
-      <c r="B7" s="25" t="s">
-        <v>108</v>
-      </c>
-      <c r="C7" s="25" t="s">
-        <v>82</v>
-      </c>
-      <c r="D7" s="26" t="n">
-        <v>5</v>
-      </c>
-      <c r="E7" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="F7" s="27" t="n">
-        <f aca="false">IF(E7="Si",N(D7),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G7" s="28" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="24" t="s">
-        <v>113</v>
-      </c>
-      <c r="B8" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="C8" s="25" t="s">
+      <c r="C6" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="D8" s="26" t="n">
-        <v>50</v>
-      </c>
-      <c r="E8" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F8" s="27" t="n">
-        <f aca="false">IF(E8="Si",N(D8),0)</f>
-        <v>50</v>
-      </c>
-      <c r="G8" s="28" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="24" t="s">
-        <v>116</v>
-      </c>
-      <c r="B9" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="C9" s="25" t="s">
-        <v>74</v>
-      </c>
-      <c r="D9" s="26" t="n">
-        <v>30</v>
-      </c>
-      <c r="E9" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F9" s="27" t="n">
-        <f aca="false">IF(E9="Si",N(D9),0)</f>
-        <v>30</v>
-      </c>
-      <c r="G9" s="28" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="24" t="s">
-        <v>117</v>
-      </c>
-      <c r="B10" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="C10" s="25" t="s">
-        <v>82</v>
-      </c>
-      <c r="D10" s="26" t="n">
-        <v>20</v>
-      </c>
-      <c r="E10" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="F10" s="27" t="n">
-        <f aca="false">IF(E10="Si",N(D10),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="28" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
-        <v>119</v>
-      </c>
-      <c r="B11" s="25" t="s">
-        <v>120</v>
-      </c>
-      <c r="C11" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="D11" s="26" t="n">
-        <v>20</v>
-      </c>
-      <c r="E11" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F11" s="27" t="n">
-        <f aca="false">IF(E11="Si",N(D11),0)</f>
-        <v>20</v>
-      </c>
-      <c r="G11" s="28" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
-        <v>122</v>
-      </c>
-      <c r="B12" s="25" t="s">
-        <v>120</v>
-      </c>
-      <c r="C12" s="25" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="26" t="n">
-        <v>10</v>
-      </c>
-      <c r="E12" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F12" s="27" t="n">
-        <f aca="false">IF(E12="Si",N(D12),0)</f>
-        <v>10</v>
-      </c>
-      <c r="G12" s="28" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24"/>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="27" t="n">
-        <f aca="false">IF(E13="Si",N(D13),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G13" s="28"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="24"/>
-      <c r="B14" s="25"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="27" t="n">
-        <f aca="false">IF(E14="Si",N(D14),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="28"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="24"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="27" t="n">
-        <f aca="false">IF(E15="Si",N(D15),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G15" s="28"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="24"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="27" t="n">
-        <f aca="false">IF(E16="Si",N(D16),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G16" s="28"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="24"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="27" t="n">
-        <f aca="false">IF(E17="Si",N(D17),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G17" s="28"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29" t="s">
-        <v>123</v>
-      </c>
-      <c r="D18" s="30" t="n">
-        <f aca="false">SUM(D5:D17)</f>
-        <v>160</v>
-      </c>
-      <c r="F18" s="30" t="n">
-        <f aca="false">SUM(F5:F17)</f>
-        <v>120</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="31" t="s">
-        <v>124</v>
-      </c>
-      <c r="B20" s="31"/>
-      <c r="C20" s="31"/>
-      <c r="D20" s="31"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="31" t="s">
-        <v>125</v>
-      </c>
-      <c r="G20" s="31"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="32" t="s">
-        <v>108</v>
-      </c>
-      <c r="F21" s="27" t="n">
-        <f aca="false">SUMIFS($F$5:$F$17,$B$5:$B$17,"Plataforma")</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="32" t="s">
-        <v>114</v>
-      </c>
-      <c r="F22" s="27" t="n">
-        <f aca="false">SUMIFS($F$5:$F$17,$B$5:$B$17,"Marketing")</f>
-        <v>80</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="F23" s="27" t="n">
-        <f aca="false">SUMIFS($F$5:$F$17,$B$5:$B$17,"Otros")</f>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="32" t="s">
-        <v>126</v>
-      </c>
-      <c r="F24" s="35" t="n">
+      <c r="D6" s="33" t="n">
         <f aca="false">Supuestos!$B$22</f>
         <v>40</v>
       </c>
-      <c r="G24" s="28" t="s">
+      <c r="E6" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" s="34" t="n">
+        <f aca="false">IF(E6="Si",N(D6),0)</f>
+        <v>40</v>
+      </c>
+      <c r="G6" s="35" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="36" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="F7" s="34" t="n">
+        <f aca="false">IF(E7="Si",N(D7),0)</f>
+        <v>10</v>
+      </c>
+      <c r="G7" s="35" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="36" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="D8" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="F8" s="34" t="n">
+        <f aca="false">IF(E8="Si",N(D8),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="35" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="36"/>
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="34" t="n">
+        <f aca="false">IF(E9="Si",N(D9),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="35"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="36"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="34" t="n">
+        <f aca="false">IF(E10="Si",N(D10),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="35"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="36"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="37"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="34" t="n">
+        <f aca="false">IF(E11="Si",N(D11),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="35"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="36"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="37"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="34" t="n">
+        <f aca="false">IF(E12="Si",N(D12),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="35"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="38" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" s="39" t="n">
+        <f aca="false">SUM(D6:D12)</f>
+        <v>65</v>
+      </c>
+      <c r="F13" s="39" t="n">
+        <f aca="false">SUM(F6:F12)</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="40" t="s">
+        <v>115</v>
+      </c>
+      <c r="B15" s="41"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="41"/>
+      <c r="G15" s="41"/>
+    </row>
+    <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="36" t="s">
+        <v>116</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D17" s="37" t="n">
+        <v>50</v>
+      </c>
+      <c r="E17" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="F17" s="34" t="n">
+        <f aca="false">IF(E17="Si",N(D17),0)</f>
+        <v>50</v>
+      </c>
+      <c r="G17" s="35" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="D18" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="F18" s="34" t="n">
+        <f aca="false">IF(E18="Si",N(D18),0)</f>
+        <v>30</v>
+      </c>
+      <c r="G18" s="35" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="D19" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="F19" s="34" t="n">
+        <f aca="false">IF(E19="Si",N(D19),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="35" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" s="34" t="n">
+        <f aca="false">IF(E20="Si",N(D20),0)</f>
+        <v>20</v>
+      </c>
+      <c r="G20" s="35" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="36" t="s">
+        <v>125</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="D21" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="F21" s="34" t="n">
+        <f aca="false">IF(E21="Si",N(D21),0)</f>
+        <v>10</v>
+      </c>
+      <c r="G21" s="35" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="36" t="s">
+        <v>126</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C22" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="D22" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="F22" s="34" t="n">
+        <f aca="false">IF(E22="Si",N(D22),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="35" t="s">
         <v>127</v>
       </c>
     </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="36"/>
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="34" t="n">
+        <f aca="false">IF(E23="Si",N(D23),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G23" s="35"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="36"/>
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="34" t="n">
+        <f aca="false">IF(E24="Si",N(D24),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="35"/>
+    </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="29" t="s">
+      <c r="A25" s="36"/>
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="34" t="n">
+        <f aca="false">IF(E25="Si",N(D25),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="35"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="36"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="37"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="34" t="n">
+        <f aca="false">IF(E26="Si",N(D26),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="35"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="38" t="s">
         <v>128</v>
       </c>
-      <c r="F25" s="30" t="n">
-        <f aca="false">SUM(F21:F24)</f>
-        <v>160</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="31" t="s">
+      <c r="D27" s="39" t="n">
+        <f aca="false">SUM(D17:D26)</f>
+        <v>135</v>
+      </c>
+      <c r="F27" s="39" t="n">
+        <f aca="false">SUM(F17:F26)</f>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="42" t="s">
         <v>129</v>
       </c>
-      <c r="B27" s="31"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="31" t="s">
-        <v>125</v>
-      </c>
-      <c r="G27" s="31"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="32" t="s">
-        <v>65</v>
-      </c>
-      <c r="F28" s="27" t="n">
-        <f aca="false">SUMIFS($F$5:$F$17,$C$5:$C$17,"Vital")</f>
-        <v>70</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="F29" s="27" t="n">
-        <f aca="false">SUMIFS($F$5:$F$17,$C$5:$C$17,"Importante")</f>
-        <v>50</v>
-      </c>
+      <c r="B29" s="43"/>
+      <c r="C29" s="43"/>
+      <c r="D29" s="43"/>
+      <c r="E29" s="43"/>
+      <c r="F29" s="43"/>
+      <c r="G29" s="43"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="32" t="s">
-        <v>82</v>
-      </c>
-      <c r="F30" s="27" t="n">
-        <f aca="false">SUMIFS($F$5:$F$17,$C$5:$C$17,"Opcional")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="38" t="s">
+      <c r="A30" s="31" t="s">
         <v>130</v>
       </c>
-      <c r="F31" s="35" t="n">
+      <c r="F30" s="33" t="n">
         <f aca="false">'Flujo de Caja'!$C$5</f>
         <v>225</v>
       </c>
+      <c r="G30" s="35" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="31" t="s">
+        <v>132</v>
+      </c>
+      <c r="F31" s="34" t="n">
+        <f aca="false">-F13</f>
+        <v>-50</v>
+      </c>
+      <c r="G31" s="35" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="29" t="s">
-        <v>131</v>
-      </c>
-      <c r="F32" s="30" t="n">
-        <f aca="false">F31-F25</f>
+      <c r="A32" s="44" t="s">
+        <v>134</v>
+      </c>
+      <c r="F32" s="39" t="n">
+        <f aca="false">F30+F31</f>
+        <v>175</v>
+      </c>
+      <c r="G32" s="35" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="31" t="s">
+        <v>136</v>
+      </c>
+      <c r="F33" s="45" t="n">
+        <f aca="false">IFERROR(F32/F30,0)</f>
+        <v>0.777777777777778</v>
+      </c>
+      <c r="G33" s="35" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="31" t="s">
+        <v>138</v>
+      </c>
+      <c r="F34" s="34" t="n">
+        <f aca="false">-F27</f>
+        <v>-110</v>
+      </c>
+      <c r="G34" s="35" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="31" t="s">
+        <v>140</v>
+      </c>
+      <c r="F35" s="34" t="n">
+        <f aca="false">F32+F34</f>
         <v>65</v>
       </c>
-      <c r="G32" s="28" t="s">
-        <v>132</v>
+      <c r="G35" s="35" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="42" t="s">
+        <v>142</v>
+      </c>
+      <c r="B37" s="43"/>
+      <c r="C37" s="43"/>
+      <c r="D37" s="43"/>
+      <c r="E37" s="43"/>
+      <c r="F37" s="43"/>
+      <c r="G37" s="43"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="F38" s="34" t="n">
+        <f aca="false">SUMIFS($F$6:$F$12,$B$6:$B$12,"Plataforma")+SUMIFS($F$17:$F$26,$B$17:$B$26,"Plataforma")</f>
+        <v>10</v>
+      </c>
+      <c r="G38" s="35" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="31" t="s">
+        <v>117</v>
+      </c>
+      <c r="F39" s="34" t="n">
+        <f aca="false">SUMIFS($F$6:$F$12,$B$6:$B$12,"Marketing")+SUMIFS($F$17:$F$26,$B$17:$B$26,"Marketing")</f>
+        <v>80</v>
+      </c>
+      <c r="G39" s="35" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="31" t="s">
+        <v>123</v>
+      </c>
+      <c r="F40" s="34" t="n">
+        <f aca="false">SUMIFS($F$6:$F$12,$B$6:$B$12,"Otros")+SUMIFS($F$17:$F$26,$B$17:$B$26,"Otros")</f>
+        <v>30</v>
+      </c>
+      <c r="G40" s="35" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="46" t="s">
+        <v>107</v>
+      </c>
+      <c r="F41" s="34" t="n">
+        <f aca="false">SUMIFS($F$6:$F$12,$B$6:$B$12,"Sueldos")</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="38" t="s">
+        <v>144</v>
+      </c>
+      <c r="F42" s="39" t="n">
+        <f aca="false">F13+F27</f>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="35" t="s">
+        <v>145</v>
+      </c>
+      <c r="F43" s="34" t="n">
+        <f aca="false">F42-SUM(F38:F41)</f>
+        <v>0</v>
+      </c>
+      <c r="G43" s="35" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="42" t="s">
+        <v>147</v>
+      </c>
+      <c r="B45" s="43"/>
+      <c r="C45" s="43"/>
+      <c r="D45" s="43"/>
+      <c r="E45" s="43"/>
+      <c r="F45" s="43"/>
+      <c r="G45" s="43"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="46" t="s">
+        <v>65</v>
+      </c>
+      <c r="F46" s="34" t="n">
+        <f aca="false">SUMIFS($F$6:$F$12,$C$6:$C$12,"Vital")+SUMIFS($F$17:$F$26,$C$17:$C$26,"Vital")</f>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="46" t="s">
+        <v>74</v>
+      </c>
+      <c r="F47" s="34" t="n">
+        <f aca="false">SUMIFS($F$6:$F$12,$C$6:$C$12,"Importante")+SUMIFS($F$17:$F$26,$C$17:$C$26,"Importante")</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="46" t="s">
+        <v>82</v>
+      </c>
+      <c r="F48" s="34" t="n">
+        <f aca="false">SUMIFS($F$6:$F$12,$C$6:$C$12,"Opcional")+SUMIFS($F$17:$F$26,$C$17:$C$26,"Opcional")</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3180,60 +3482,49 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="C5:C17">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+  <conditionalFormatting sqref="C6:C12">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>"Vital"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>"Importante"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>"Opcional"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A28">
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+  <conditionalFormatting sqref="C17:C26">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>"Vital"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>"Importante"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>"Opcional"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A29">
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+  <conditionalFormatting sqref="A46:A48">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>"Vital"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>"Importante"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
-      <formula>"Opcional"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A30">
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>"Vital"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>"Importante"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="13" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>"Opcional"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B17" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B7:B12 B17:B26" type="list">
       <formula1>"Plataforma,Marketing,Otros"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C17" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C6:C12 C17:C26" type="list">
       <formula1>"Vital,Importante,Opcional"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E17" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E7:E12 E17:E26" type="list">
       <formula1>"Si,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3262,7 +3553,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>133</v>
+        <v>148</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3277,62 +3568,62 @@
         <v>45</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>139</v>
+        <v>154</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="B4" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="39" t="n">
+      <c r="C4" s="47" t="n">
         <f aca="false">MIN(Supuestos!$B$21,Supuestos!$B$5)</f>
         <v>15</v>
       </c>
-      <c r="D4" s="39" t="n">
+      <c r="D4" s="47" t="n">
         <f aca="false">MIN(Supuestos!$B$21,ROUND(C4*(1+Supuestos!$B$6),0))</f>
         <v>15</v>
       </c>
-      <c r="E4" s="39" t="n">
+      <c r="E4" s="47" t="n">
         <f aca="false">MIN(Supuestos!$B$21,ROUND(D4*(1+Supuestos!$B$6),0))</f>
         <v>15</v>
       </c>
-      <c r="F4" s="39" t="n">
+      <c r="F4" s="47" t="n">
         <f aca="false">MIN(Supuestos!$B$21,ROUND(E4*(1+Supuestos!$B$6),0))</f>
         <v>15</v>
       </c>
-      <c r="G4" s="39" t="n">
+      <c r="G4" s="47" t="n">
         <f aca="false">MIN(Supuestos!$B$21,ROUND(F4*(1+Supuestos!$B$6),0))</f>
         <v>15</v>
       </c>
-      <c r="H4" s="39" t="n">
+      <c r="H4" s="47" t="n">
         <f aca="false">MIN(Supuestos!$B$21,ROUND(G4*(1+Supuestos!$B$6),0))</f>
         <v>15</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="B5" s="13" t="n">
         <v>0</v>
@@ -3364,7 +3655,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="B6" s="13" t="n">
         <v>0</v>
@@ -3395,8 +3686,8 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="40" t="s">
-        <v>144</v>
+      <c r="A7" s="27" t="s">
+        <v>159</v>
       </c>
       <c r="B7" s="13" t="n">
         <v>0</v>
@@ -3428,7 +3719,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="B8" s="13" t="n">
         <v>0</v>
@@ -3460,7 +3751,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>146</v>
+        <v>161</v>
       </c>
       <c r="B9" s="13" t="n">
         <v>0</v>
@@ -3492,7 +3783,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>147</v>
+        <v>162</v>
       </c>
       <c r="B10" s="13" t="n">
         <v>0</v>
@@ -3524,7 +3815,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="B11" s="13" t="n">
         <v>0</v>
@@ -3555,8 +3846,8 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="40" t="s">
-        <v>149</v>
+      <c r="A12" s="27" t="s">
+        <v>164</v>
       </c>
       <c r="B12" s="13" t="n">
         <v>0</v>
@@ -3587,8 +3878,8 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="40" t="s">
-        <v>150</v>
+      <c r="A13" s="27" t="s">
+        <v>165</v>
       </c>
       <c r="B13" s="13" t="n">
         <v>0</v>
@@ -3620,7 +3911,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>151</v>
+        <v>166</v>
       </c>
       <c r="B14" s="13" t="n">
         <v>0</v>
@@ -3652,7 +3943,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>152</v>
+        <v>167</v>
       </c>
       <c r="B15" s="13" t="n">
         <v>0</v>
@@ -3684,7 +3975,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">-Inversion!$B$13</f>
@@ -3710,74 +4001,74 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="41" t="s">
-        <v>154</v>
-      </c>
-      <c r="B17" s="22" t="n">
+      <c r="A17" s="48" t="s">
+        <v>169</v>
+      </c>
+      <c r="B17" s="19" t="n">
         <f aca="false">B15+B16</f>
         <v>-88</v>
       </c>
-      <c r="C17" s="22" t="n">
+      <c r="C17" s="19" t="n">
         <f aca="false">C15+C16</f>
         <v>47.45</v>
       </c>
-      <c r="D17" s="22" t="n">
+      <c r="D17" s="19" t="n">
         <f aca="false">D15+D16</f>
         <v>47.45</v>
       </c>
-      <c r="E17" s="22" t="n">
+      <c r="E17" s="19" t="n">
         <f aca="false">E15+E16</f>
         <v>47.45</v>
       </c>
-      <c r="F17" s="22" t="n">
+      <c r="F17" s="19" t="n">
         <f aca="false">F15+F16</f>
         <v>47.45</v>
       </c>
-      <c r="G17" s="22" t="n">
+      <c r="G17" s="19" t="n">
         <f aca="false">G15+G16</f>
         <v>47.45</v>
       </c>
-      <c r="H17" s="22" t="n">
+      <c r="H17" s="19" t="n">
         <f aca="false">H15+H16</f>
         <v>47.45</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="41" t="s">
-        <v>155</v>
-      </c>
-      <c r="B18" s="22" t="n">
+      <c r="A18" s="48" t="s">
+        <v>170</v>
+      </c>
+      <c r="B18" s="19" t="n">
         <f aca="false">B17</f>
         <v>-88</v>
       </c>
-      <c r="C18" s="22" t="n">
+      <c r="C18" s="19" t="n">
         <f aca="false">B18+C17</f>
         <v>-40.55</v>
       </c>
-      <c r="D18" s="22" t="n">
+      <c r="D18" s="19" t="n">
         <f aca="false">C18+D17</f>
         <v>6.90000000000001</v>
       </c>
-      <c r="E18" s="22" t="n">
+      <c r="E18" s="19" t="n">
         <f aca="false">D18+E17</f>
         <v>54.35</v>
       </c>
-      <c r="F18" s="22" t="n">
+      <c r="F18" s="19" t="n">
         <f aca="false">E18+F17</f>
         <v>101.8</v>
       </c>
-      <c r="G18" s="22" t="n">
+      <c r="G18" s="19" t="n">
         <f aca="false">F18+G17</f>
         <v>149.25</v>
       </c>
-      <c r="H18" s="22" t="n">
+      <c r="H18" s="19" t="n">
         <f aca="false">G18+H17</f>
         <v>196.7</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -3810,240 +4101,240 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>159</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
+        <v>175</v>
+      </c>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">Inversion!$B$13</f>
         <v>88</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>162</v>
+        <v>177</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">MAX(0,-MIN('Flujo de Caja'!$B$18:$H$18)-Inversion!$B$13)</f>
         <v>0</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="40" t="s">
-        <v>165</v>
-      </c>
-      <c r="B7" s="22" t="n">
+      <c r="A7" s="27" t="s">
+        <v>180</v>
+      </c>
+      <c r="B7" s="19" t="n">
         <f aca="false">MAX(0,-MIN('Flujo de Caja'!$B$18:$H$18))</f>
         <v>88</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>166</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="B8" s="42"/>
-      <c r="C8" s="42"/>
+        <v>182</v>
+      </c>
+      <c r="B8" s="25"/>
+      <c r="C8" s="25"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="B9" s="13" t="n">
         <f aca="false">NPV(Supuestos!$B$20,'Flujo de Caja'!$C$17:$H$17)+'Flujo de Caja'!$B$17</f>
         <v>187.479126512871</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>169</v>
+        <v>184</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B10" s="43" t="n">
+        <v>185</v>
+      </c>
+      <c r="B10" s="49" t="n">
         <f aca="false">IFERROR(IRR('Flujo de Caja'!$B$17:$H$17,0.02),"No calculable")</f>
         <v>0.489910783440648</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="B11" s="43" t="n">
+        <v>187</v>
+      </c>
+      <c r="B11" s="49" t="n">
         <f aca="false">IFERROR((1+B10)^12-1,"No calculable")</f>
         <v>118.652881325872</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>173</v>
+        <v>188</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="B12" s="44" t="n">
+        <v>189</v>
+      </c>
+      <c r="B12" s="50" t="n">
         <f aca="false">Supuestos!$B$17</f>
         <v>0.12</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false" t="array" ref="B13:B13">IF(INDEX('Flujo de Caja'!$B$18:$H$18,1,COLUMNS('Flujo de Caja'!$B$18:$H$18))&lt;0,"No recupera en 6 meses",COUNTIF('Flujo de Caja'!$B$18:$H$18,"&lt;0"))</f>
         <v>2</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="B14" s="13" t="n">
         <f aca="false" t="array" ref="B14:B14">INDEX('Flujo de Caja'!$B$18:$H$18,1,COLUMNS('Flujo de Caja'!$B$18:$H$18))</f>
         <v>196.7</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B15" s="43" t="n">
+        <v>195</v>
+      </c>
+      <c r="B15" s="49" t="n">
         <f aca="false">IFERROR(B14/B7,0)</f>
         <v>2.23522727272727</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>182</v>
-      </c>
-      <c r="B16" s="42"/>
-      <c r="C16" s="42"/>
+        <v>197</v>
+      </c>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">ROUNDUP(Supuestos!$B$23/Supuestos!$B$24,0)</f>
         <v>11</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="B18" s="39" t="n">
+        <v>200</v>
+      </c>
+      <c r="B18" s="47" t="n">
         <f aca="false">Supuestos!$B$21</f>
         <v>15</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="B19" s="9" t="n">
         <f aca="false">B17*Supuestos!$B$4</f>
         <v>165</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="B20" s="9" t="n">
         <f aca="false">B18*Supuestos!$B$24-Supuestos!$B$23</f>
         <v>65</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="B21" s="43" t="n">
+        <v>206</v>
+      </c>
+      <c r="B21" s="49" t="n">
         <f aca="false">IFERROR(B20/(B18*Supuestos!$B$4),0)</f>
         <v>0.288888888888889</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>193</v>
-      </c>
-      <c r="B22" s="42"/>
-      <c r="C22" s="42"/>
+        <v>208</v>
+      </c>
+      <c r="B22" s="25"/>
+      <c r="C22" s="25"/>
     </row>
     <row r="23" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="B23" s="45" t="str">
+        <v>209</v>
+      </c>
+      <c r="B23" s="51" t="str">
         <f aca="false">IF(AND(ISNUMBER(B9),B9&gt;0,B18&gt;=B17),"VIABLE: VAN positivo y la capacidad supera el punto de equilibrio",IF(B18&lt;B17,"NO VIABLE: la capacidad no alcanza el punto de equilibrio","NO VIABLE en 6 meses: VAN negativo"))</f>
         <v>VIABLE: VAN positivo y la capacidad supera el punto de equilibrio</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -4074,7 +4365,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4092,99 +4383,99 @@
       <c r="O1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23" t="s">
-        <v>197</v>
-      </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
+      <c r="A2" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="20"/>
+      <c r="M2" s="20"/>
+      <c r="N2" s="20"/>
+      <c r="O2" s="20"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="40" t="s">
-        <v>198</v>
-      </c>
-      <c r="B4" s="22" t="n">
+      <c r="A4" s="27" t="s">
+        <v>213</v>
+      </c>
+      <c r="B4" s="19" t="n">
         <f aca="false">F14</f>
         <v>1048</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="40" t="s">
-        <v>199</v>
-      </c>
-      <c r="B5" s="46" t="n">
+      <c r="A5" s="27" t="s">
+        <v>214</v>
+      </c>
+      <c r="B5" s="52" t="n">
         <f aca="false">COUNT(D9:D14)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>202</v>
+        <v>217</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>204</v>
+        <v>219</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>208</v>
+        <v>223</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>209</v>
+        <v>224</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>211</v>
+        <v>226</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>213</v>
+        <v>228</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>214</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="47" t="n">
+      <c r="A9" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="B9" s="43" t="n">
+      <c r="B9" s="49" t="n">
         <f aca="false">F9/$B$4</f>
         <v>0.236641221374046</v>
       </c>
       <c r="C9" s="8"/>
-      <c r="D9" s="48"/>
+      <c r="D9" s="23"/>
       <c r="E9" s="9" t="n">
         <f aca="false">-'Flujo de Caja'!C12+Inversion!$B$13</f>
         <v>248</v>
@@ -4205,11 +4496,11 @@
         <f aca="false">IF(D9="","",G9-F9)</f>
         <v/>
       </c>
-      <c r="J9" s="49" t="str">
+      <c r="J9" s="54" t="str">
         <f aca="false">IF(D9="","",IFERROR(G9/D9,0))</f>
         <v/>
       </c>
-      <c r="K9" s="49" t="str">
+      <c r="K9" s="54" t="str">
         <f aca="false">IF(D9="","",IFERROR(G9/F9,0))</f>
         <v/>
       </c>
@@ -4225,21 +4516,21 @@
         <f aca="false">IF(D9="","",$B$4-L9)</f>
         <v/>
       </c>
-      <c r="O9" s="49" t="str">
+      <c r="O9" s="54" t="str">
         <f aca="false">IF(D9="","",IFERROR(($B$4-G9)/($B$4-D9),0))</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="47" t="n">
+      <c r="A10" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="B10" s="43" t="n">
+      <c r="B10" s="49" t="n">
         <f aca="false">F10/$B$4</f>
         <v>0.389312977099237</v>
       </c>
       <c r="C10" s="8"/>
-      <c r="D10" s="48"/>
+      <c r="D10" s="23"/>
       <c r="E10" s="9" t="n">
         <f aca="false">-'Flujo de Caja'!D12</f>
         <v>160</v>
@@ -4260,11 +4551,11 @@
         <f aca="false">IF(D10="","",G10-F10)</f>
         <v/>
       </c>
-      <c r="J10" s="49" t="str">
+      <c r="J10" s="54" t="str">
         <f aca="false">IF(D10="","",IFERROR(G10/D10,0))</f>
         <v/>
       </c>
-      <c r="K10" s="49" t="str">
+      <c r="K10" s="54" t="str">
         <f aca="false">IF(D10="","",IFERROR(G10/F10,0))</f>
         <v/>
       </c>
@@ -4280,21 +4571,21 @@
         <f aca="false">IF(D10="","",$B$4-L10)</f>
         <v/>
       </c>
-      <c r="O10" s="49" t="str">
+      <c r="O10" s="54" t="str">
         <f aca="false">IF(D10="","",IFERROR(($B$4-G10)/($B$4-D10),0))</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="47" t="n">
+      <c r="A11" s="53" t="n">
         <v>3</v>
       </c>
-      <c r="B11" s="43" t="n">
+      <c r="B11" s="49" t="n">
         <f aca="false">F11/$B$4</f>
         <v>0.541984732824428</v>
       </c>
       <c r="C11" s="8"/>
-      <c r="D11" s="48"/>
+      <c r="D11" s="23"/>
       <c r="E11" s="9" t="n">
         <f aca="false">-'Flujo de Caja'!E12</f>
         <v>160</v>
@@ -4315,11 +4606,11 @@
         <f aca="false">IF(D11="","",G11-F11)</f>
         <v/>
       </c>
-      <c r="J11" s="49" t="str">
+      <c r="J11" s="54" t="str">
         <f aca="false">IF(D11="","",IFERROR(G11/D11,0))</f>
         <v/>
       </c>
-      <c r="K11" s="49" t="str">
+      <c r="K11" s="54" t="str">
         <f aca="false">IF(D11="","",IFERROR(G11/F11,0))</f>
         <v/>
       </c>
@@ -4335,21 +4626,21 @@
         <f aca="false">IF(D11="","",$B$4-L11)</f>
         <v/>
       </c>
-      <c r="O11" s="49" t="str">
+      <c r="O11" s="54" t="str">
         <f aca="false">IF(D11="","",IFERROR(($B$4-G11)/($B$4-D11),0))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="47" t="n">
+      <c r="A12" s="53" t="n">
         <v>4</v>
       </c>
-      <c r="B12" s="43" t="n">
+      <c r="B12" s="49" t="n">
         <f aca="false">F12/$B$4</f>
         <v>0.694656488549618</v>
       </c>
       <c r="C12" s="8"/>
-      <c r="D12" s="48"/>
+      <c r="D12" s="23"/>
       <c r="E12" s="9" t="n">
         <f aca="false">-'Flujo de Caja'!F12</f>
         <v>160</v>
@@ -4370,11 +4661,11 @@
         <f aca="false">IF(D12="","",G12-F12)</f>
         <v/>
       </c>
-      <c r="J12" s="49" t="str">
+      <c r="J12" s="54" t="str">
         <f aca="false">IF(D12="","",IFERROR(G12/D12,0))</f>
         <v/>
       </c>
-      <c r="K12" s="49" t="str">
+      <c r="K12" s="54" t="str">
         <f aca="false">IF(D12="","",IFERROR(G12/F12,0))</f>
         <v/>
       </c>
@@ -4390,21 +4681,21 @@
         <f aca="false">IF(D12="","",$B$4-L12)</f>
         <v/>
       </c>
-      <c r="O12" s="49" t="str">
+      <c r="O12" s="54" t="str">
         <f aca="false">IF(D12="","",IFERROR(($B$4-G12)/($B$4-D12),0))</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="47" t="n">
+      <c r="A13" s="53" t="n">
         <v>5</v>
       </c>
-      <c r="B13" s="43" t="n">
+      <c r="B13" s="49" t="n">
         <f aca="false">F13/$B$4</f>
         <v>0.847328244274809</v>
       </c>
       <c r="C13" s="8"/>
-      <c r="D13" s="48"/>
+      <c r="D13" s="23"/>
       <c r="E13" s="9" t="n">
         <f aca="false">-'Flujo de Caja'!G12</f>
         <v>160</v>
@@ -4425,11 +4716,11 @@
         <f aca="false">IF(D13="","",G13-F13)</f>
         <v/>
       </c>
-      <c r="J13" s="49" t="str">
+      <c r="J13" s="54" t="str">
         <f aca="false">IF(D13="","",IFERROR(G13/D13,0))</f>
         <v/>
       </c>
-      <c r="K13" s="49" t="str">
+      <c r="K13" s="54" t="str">
         <f aca="false">IF(D13="","",IFERROR(G13/F13,0))</f>
         <v/>
       </c>
@@ -4445,21 +4736,21 @@
         <f aca="false">IF(D13="","",$B$4-L13)</f>
         <v/>
       </c>
-      <c r="O13" s="49" t="str">
+      <c r="O13" s="54" t="str">
         <f aca="false">IF(D13="","",IFERROR(($B$4-G13)/($B$4-D13),0))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="47" t="n">
+      <c r="A14" s="53" t="n">
         <v>6</v>
       </c>
-      <c r="B14" s="43" t="n">
+      <c r="B14" s="49" t="n">
         <f aca="false">F14/$B$4</f>
         <v>1</v>
       </c>
       <c r="C14" s="8"/>
-      <c r="D14" s="48"/>
+      <c r="D14" s="23"/>
       <c r="E14" s="9" t="n">
         <f aca="false">-'Flujo de Caja'!H12</f>
         <v>160</v>
@@ -4480,11 +4771,11 @@
         <f aca="false">IF(D14="","",G14-F14)</f>
         <v/>
       </c>
-      <c r="J14" s="49" t="str">
+      <c r="J14" s="54" t="str">
         <f aca="false">IF(D14="","",IFERROR(G14/D14,0))</f>
         <v/>
       </c>
-      <c r="K14" s="49" t="str">
+      <c r="K14" s="54" t="str">
         <f aca="false">IF(D14="","",IFERROR(G14/F14,0))</f>
         <v/>
       </c>
@@ -4500,164 +4791,164 @@
         <f aca="false">IF(D14="","",$B$4-L14)</f>
         <v/>
       </c>
-      <c r="O14" s="49" t="str">
+      <c r="O14" s="54" t="str">
         <f aca="false">IF(D14="","",IFERROR(($B$4-G14)/($B$4-D14),0))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>215</v>
-      </c>
-      <c r="B16" s="42"/>
-      <c r="C16" s="42"/>
+        <v>230</v>
+      </c>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>216</v>
+        <v>231</v>
       </c>
       <c r="B17" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(F9:F14,$B$5))</f>
         <v>Sin datos</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>217</v>
+        <v>232</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
       <c r="B18" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(G9:G14,$B$5))</f>
         <v>Sin datos</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>218</v>
+        <v>233</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>219</v>
+        <v>234</v>
       </c>
       <c r="B19" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(D9:D14,$B$5))</f>
         <v>Sin datos</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>220</v>
+        <v>235</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>221</v>
+        <v>236</v>
       </c>
       <c r="B20" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(H9:H14,$B$5))</f>
         <v>Sin datos</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>223</v>
+        <v>238</v>
       </c>
       <c r="B21" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(I9:I14,$B$5))</f>
         <v>Sin datos</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="B22" s="49" t="str">
+        <v>240</v>
+      </c>
+      <c r="B22" s="54" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(J9:J14,$B$5))</f>
         <v>Sin datos</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>226</v>
+        <v>241</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="B23" s="49" t="str">
+        <v>242</v>
+      </c>
+      <c r="B23" s="54" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(K9:K14,$B$5))</f>
         <v>Sin datos</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>228</v>
+        <v>243</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>229</v>
+        <v>244</v>
       </c>
       <c r="B24" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(L9:L14,$B$5))</f>
         <v>Sin datos</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>230</v>
+        <v>245</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>231</v>
+        <v>246</v>
       </c>
       <c r="B25" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(M9:M14,$B$5))</f>
         <v>Sin datos</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>232</v>
+        <v>247</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
       <c r="B26" s="13" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(N9:N14,$B$5))</f>
         <v>Sin datos</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>234</v>
+        <v>249</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>235</v>
-      </c>
-      <c r="B27" s="49" t="str">
+        <v>250</v>
+      </c>
+      <c r="B27" s="54" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",INDEX(O9:O14,$B$5))</f>
         <v>Sin datos</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="19" t="s">
-        <v>237</v>
-      </c>
-      <c r="B28" s="40" t="str">
+      <c r="A28" s="17" t="s">
+        <v>252</v>
+      </c>
+      <c r="B28" s="27" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",IF(B22&gt;=1,"Bajo presupuesto","Sobre presupuesto"))</f>
         <v>Sin datos</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="19" t="s">
-        <v>238</v>
-      </c>
-      <c r="B29" s="40" t="str">
+      <c r="A29" s="17" t="s">
+        <v>253</v>
+      </c>
+      <c r="B29" s="27" t="str">
         <f aca="false">IF($B$5=0,"Sin datos",IF(B23&gt;=1,"Adelantado / a tiempo","Atrasado"))</f>
         <v>Sin datos</v>
       </c>

</xml_diff>